<commit_message>
Ajusta fontes de avaliacao de evidencias
</commit_message>
<xml_diff>
--- a/02-Execucao/01-Questionario/04-Resultados_iGovTI/20260621-iGovTI-2026-Ajustado-Comparavel.xlsx
+++ b/02-Execucao/01-Questionario/04-Resultados_iGovTI/20260621-iGovTI-2026-Ajustado-Comparavel.xlsx
@@ -829,7 +829,7 @@
         <v>20</v>
       </c>
       <c r="B2">
-        <v>0.008257613705133999</v>
+        <v>0.004894582405871045</v>
       </c>
       <c r="C2" t="s">
         <v>134</v>
@@ -865,22 +865,22 @@
         <v>0</v>
       </c>
       <c r="N2">
-        <v>0.07471246994259101</v>
+        <v>0.06983033213692173</v>
       </c>
       <c r="O2">
-        <v>0.2666666666666667</v>
+        <v>0.1500000000000001</v>
       </c>
       <c r="P2">
         <v>0</v>
       </c>
       <c r="Q2">
-        <v>0.01916095325953799</v>
+        <v>0.01790886757192877</v>
       </c>
       <c r="R2">
-        <v>0.04483827683268945</v>
+        <v>0.02657724722075695</v>
       </c>
       <c r="S2">
-        <v>0.016515227410268</v>
+        <v>0.00978916481174209</v>
       </c>
       <c r="T2">
         <v>0.1249239775786869</v>
@@ -891,13 +891,13 @@
         <v>21</v>
       </c>
       <c r="B3">
-        <v>0.1965338949042437</v>
+        <v>0.09506818522245383</v>
       </c>
       <c r="C3" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="D3">
-        <v>0.2444444444444445</v>
+        <v>0</v>
       </c>
       <c r="E3">
         <v>0.01199770569238325</v>
@@ -906,13 +906,13 @@
         <v>0.5</v>
       </c>
       <c r="G3">
-        <v>0.2444295548303219</v>
+        <v>0.160711053811857</v>
       </c>
       <c r="H3">
-        <v>0.20625</v>
+        <v>0.025</v>
       </c>
       <c r="I3">
-        <v>0.2080747166913506</v>
+        <v>0.02429690983669855</v>
       </c>
       <c r="J3">
         <v>0.0381845691462976</v>
@@ -927,7 +927,7 @@
         <v>0.05</v>
       </c>
       <c r="N3">
-        <v>0.245373376317999</v>
+        <v>0.02481049554247315</v>
       </c>
       <c r="O3">
         <v>0.05</v>
@@ -936,16 +936,16 @@
         <v>0.05</v>
       </c>
       <c r="Q3">
-        <v>0.09232006450052971</v>
+        <v>0.03575393768694281</v>
       </c>
       <c r="R3">
-        <v>0.04834389832956001</v>
+        <v>0.03758952374296143</v>
       </c>
       <c r="S3">
-        <v>0.1486382349781654</v>
+        <v>0.02942531663305064</v>
       </c>
       <c r="T3">
-        <v>0.943161015845023</v>
+        <v>0</v>
       </c>
     </row>
     <row r="4" spans="1:20">
@@ -1015,7 +1015,7 @@
         <v>23</v>
       </c>
       <c r="B5">
-        <v>0.2379973088528159</v>
+        <v>0.1662028075839953</v>
       </c>
       <c r="C5" t="s">
         <v>135</v>
@@ -1027,13 +1027,13 @@
         <v>0</v>
       </c>
       <c r="F5">
-        <v>0.2714285714285715</v>
+        <v>0</v>
       </c>
       <c r="G5">
-        <v>0.1363730550198272</v>
+        <v>0.051372716534058</v>
       </c>
       <c r="H5">
-        <v>0.51125</v>
+        <v>0.3412500000000001</v>
       </c>
       <c r="I5">
         <v>0.1793967191405526</v>
@@ -1048,10 +1048,10 @@
         <v>0.26350964164875</v>
       </c>
       <c r="M5">
-        <v>0.3020156368703212</v>
+        <v>0.2546719542810709</v>
       </c>
       <c r="N5">
-        <v>0.2946664042540086</v>
+        <v>0.2005108894303867</v>
       </c>
       <c r="O5">
         <v>0.5</v>
@@ -1060,16 +1060,16 @@
         <v>0</v>
       </c>
       <c r="Q5">
-        <v>0.2737597705155187</v>
+        <v>0.2393773735977918</v>
       </c>
       <c r="R5">
-        <v>0.3166523355879047</v>
+        <v>0.3101155405752836</v>
       </c>
       <c r="S5">
-        <v>0.3396215626858046</v>
+        <v>0.2810328986339327</v>
       </c>
       <c r="T5">
-        <v>0.7401710112919844</v>
+        <v>0.6549125350595204</v>
       </c>
     </row>
     <row r="6" spans="1:20">
@@ -1077,13 +1077,13 @@
         <v>24</v>
       </c>
       <c r="B6">
-        <v>0.2155751060140498</v>
+        <v>0.1074908829895896</v>
       </c>
       <c r="C6" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="D6">
-        <v>0.4333333333333333</v>
+        <v>0</v>
       </c>
       <c r="E6">
         <v>0</v>
@@ -1092,16 +1092,16 @@
         <v>0.05</v>
       </c>
       <c r="G6">
-        <v>0.1640680270767625</v>
+        <v>0.0156579570894838</v>
       </c>
       <c r="H6">
-        <v>0.49</v>
+        <v>0.32</v>
       </c>
       <c r="I6">
         <v>0.1028930682242935</v>
       </c>
       <c r="J6">
-        <v>0.2086374417506965</v>
+        <v>0.03976466684964675</v>
       </c>
       <c r="K6">
         <v>0</v>
@@ -1125,10 +1125,10 @@
         <v>0.171280569812873</v>
       </c>
       <c r="R6">
-        <v>0.2013362129116579</v>
+        <v>0.1699039638216397</v>
       </c>
       <c r="S6">
-        <v>0.2670821849513371</v>
+        <v>0.1993238088896953</v>
       </c>
       <c r="T6">
         <v>0.1249239775786869</v>
@@ -1139,7 +1139,7 @@
         <v>25</v>
       </c>
       <c r="B7">
-        <v>0.2322698175147301</v>
+        <v>0.1690302682310862</v>
       </c>
       <c r="C7" t="s">
         <v>135</v>
@@ -1157,13 +1157,13 @@
         <v>0.156579570894838</v>
       </c>
       <c r="H7">
-        <v>0.5</v>
+        <v>0.33</v>
       </c>
       <c r="I7">
-        <v>0.2601786586960324</v>
+        <v>0.0546948617719611</v>
       </c>
       <c r="J7">
-        <v>0.2401332448591994</v>
+        <v>0.1500000000000001</v>
       </c>
       <c r="K7">
         <v>0.15</v>
@@ -1175,7 +1175,7 @@
         <v>0.9426717283081794</v>
       </c>
       <c r="N7">
-        <v>0.4632838747962885</v>
+        <v>0.3392146750823997</v>
       </c>
       <c r="O7">
         <v>0</v>
@@ -1184,16 +1184,16 @@
         <v>0.15</v>
       </c>
       <c r="Q7">
-        <v>0.3572760685682754</v>
+        <v>0.3254569607474149</v>
       </c>
       <c r="R7">
-        <v>0.1747281826044822</v>
+        <v>0.1519022418889608</v>
       </c>
       <c r="S7">
-        <v>0.3079600641346223</v>
+        <v>0.1814809655673344</v>
       </c>
       <c r="T7">
-        <v>0.999999999999999</v>
+        <v>0.9147415237675349</v>
       </c>
     </row>
     <row r="8" spans="1:20">
@@ -1201,7 +1201,7 @@
         <v>26</v>
       </c>
       <c r="B8">
-        <v>0.1171164432816861</v>
+        <v>0.1103312074940714</v>
       </c>
       <c r="C8" t="s">
         <v>134</v>
@@ -1222,7 +1222,7 @@
         <v>0.075</v>
       </c>
       <c r="I8">
-        <v>0.122821443348241</v>
+        <v>0.07776599528314995</v>
       </c>
       <c r="J8">
         <v>0.1145537074388928</v>
@@ -1252,7 +1252,7 @@
         <v>0.1675484985128222</v>
       </c>
       <c r="S8">
-        <v>0.1234918500098057</v>
+        <v>0.1099213784345764</v>
       </c>
       <c r="T8">
         <v>0.1499999999999999</v>
@@ -1263,7 +1263,7 @@
         <v>27</v>
       </c>
       <c r="B9">
-        <v>0.3621637105340755</v>
+        <v>0.2524863137063363</v>
       </c>
       <c r="C9" t="s">
         <v>135</v>
@@ -1281,13 +1281,13 @@
         <v>0.1905719605161478</v>
       </c>
       <c r="H9">
-        <v>1</v>
+        <v>0.6174999999999999</v>
       </c>
       <c r="I9">
-        <v>0.4322918268613428</v>
+        <v>0.1670031774765376</v>
       </c>
       <c r="J9">
-        <v>0.2835273103868767</v>
+        <v>0.1146545354858269</v>
       </c>
       <c r="K9">
         <v>0.15</v>
@@ -1299,7 +1299,7 @@
         <v>0.7379575407672525</v>
       </c>
       <c r="N9">
-        <v>0.2282992325914181</v>
+        <v>0.1466361105107093</v>
       </c>
       <c r="O9">
         <v>0.15</v>
@@ -1308,16 +1308,16 @@
         <v>0.15</v>
       </c>
       <c r="Q9">
-        <v>0.2738311819522368</v>
+        <v>0.2528876464698902</v>
       </c>
       <c r="R9">
-        <v>0.19839623994975</v>
+        <v>0.1629821975422021</v>
       </c>
       <c r="S9">
-        <v>0.5337554605520032</v>
+        <v>0.3144006668965248</v>
       </c>
       <c r="T9">
-        <v>0.441489281016936</v>
+        <v>0.02507602242131295</v>
       </c>
     </row>
     <row r="10" spans="1:20">
@@ -1325,7 +1325,7 @@
         <v>28</v>
       </c>
       <c r="B10">
-        <v>0.04803246354110126</v>
+        <v>0.04785710440082451</v>
       </c>
       <c r="C10" t="s">
         <v>134</v>
@@ -1361,7 +1361,7 @@
         <v>0.1591957468445924</v>
       </c>
       <c r="N10">
-        <v>0.1792928268340157</v>
+        <v>0.1597642756113385</v>
       </c>
       <c r="O10">
         <v>0</v>
@@ -1370,13 +1370,13 @@
         <v>0.2375</v>
       </c>
       <c r="Q10">
-        <v>0.08039775585013657</v>
+        <v>0.07538941309969968</v>
       </c>
       <c r="R10">
-        <v>0.1102937294027784</v>
+        <v>0.1093415412818951</v>
       </c>
       <c r="S10">
-        <v>0.09606492708220252</v>
+        <v>0.09571420880164902</v>
       </c>
       <c r="T10">
         <v>0.1499999999999999</v>
@@ -1387,25 +1387,25 @@
         <v>29</v>
       </c>
       <c r="B11">
-        <v>0.4185188357855134</v>
+        <v>0.2344479453065925</v>
       </c>
       <c r="C11" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="D11">
-        <v>0.6222222222222222</v>
+        <v>0.5277777777777778</v>
       </c>
       <c r="E11">
         <v>0.4163925873059408</v>
       </c>
       <c r="F11">
-        <v>0.8785714285714286</v>
+        <v>0</v>
       </c>
       <c r="G11">
-        <v>0.6316216331824059</v>
+        <v>0.3241431741256408</v>
       </c>
       <c r="H11">
-        <v>0.325</v>
+        <v>0.15</v>
       </c>
       <c r="I11">
         <v>0.1500000000000001</v>
@@ -1423,7 +1423,7 @@
         <v>0.15</v>
       </c>
       <c r="N11">
-        <v>0.2715916694017477</v>
+        <v>0.1140146693316767</v>
       </c>
       <c r="O11">
         <v>0.15</v>
@@ -1432,13 +1432,13 @@
         <v>0.15</v>
       </c>
       <c r="Q11">
-        <v>0.2175418526114568</v>
+        <v>0.1771292476548693</v>
       </c>
       <c r="R11">
-        <v>0.1434370655335953</v>
+        <v>0.135753804963968</v>
       </c>
       <c r="S11">
-        <v>0.2054160383886208</v>
+        <v>0.1447527164875443</v>
       </c>
       <c r="T11">
         <v>0.1249239775786869</v>
@@ -1449,7 +1449,7 @@
         <v>30</v>
       </c>
       <c r="B12">
-        <v>0.2261085807987455</v>
+        <v>0.2161581179345408</v>
       </c>
       <c r="C12" t="s">
         <v>135</v>
@@ -1473,10 +1473,10 @@
         <v>0.2328160824998445</v>
       </c>
       <c r="J12">
-        <v>0.2839082163419612</v>
+        <v>0.1145537074388928</v>
       </c>
       <c r="K12">
-        <v>0.15</v>
+        <v>0</v>
       </c>
       <c r="L12">
         <v>0.1499999999985</v>
@@ -1497,10 +1497,10 @@
         <v>0.1784133086891351</v>
       </c>
       <c r="R12">
-        <v>0.1803262537693739</v>
+        <v>0.1262959219507256</v>
       </c>
       <c r="S12">
-        <v>0.3757246027332967</v>
+        <v>0.3558236770048872</v>
       </c>
       <c r="T12">
         <v>0.1499999999999999</v>
@@ -1511,7 +1511,7 @@
         <v>31</v>
       </c>
       <c r="B13">
-        <v>0.1039769420581566</v>
+        <v>0.1016007063410602</v>
       </c>
       <c r="C13" t="s">
         <v>134</v>
@@ -1535,7 +1535,7 @@
         <v>0.0300023387141979</v>
       </c>
       <c r="J13">
-        <v>0.1688727749010497</v>
+        <v>0.1021091197076115</v>
       </c>
       <c r="K13">
         <v>0</v>
@@ -1547,7 +1547,7 @@
         <v>0.05058376913984175</v>
       </c>
       <c r="N13">
-        <v>0.05719075715212587</v>
+        <v>0.0474264815407873</v>
       </c>
       <c r="O13">
         <v>0.15</v>
@@ -1556,13 +1556,13 @@
         <v>0.5</v>
       </c>
       <c r="Q13">
-        <v>0.02560278014780605</v>
+        <v>0.0230986087725876</v>
       </c>
       <c r="R13">
-        <v>0.1426244107096823</v>
+        <v>0.1297216135206288</v>
       </c>
       <c r="S13">
-        <v>0.1565811675822552</v>
+        <v>0.1518286961480624</v>
       </c>
       <c r="T13">
         <v>0</v>
@@ -1573,7 +1573,7 @@
         <v>32</v>
       </c>
       <c r="B14">
-        <v>0.5758853687284125</v>
+        <v>0.5240335722349011</v>
       </c>
       <c r="C14" t="s">
         <v>136</v>
@@ -1591,16 +1591,16 @@
         <v>0.5822001235257146</v>
       </c>
       <c r="H14">
-        <v>1</v>
+        <v>0.8087500000000001</v>
       </c>
       <c r="I14">
         <v>0.1500000000000001</v>
       </c>
       <c r="J14">
-        <v>0.4626191233923148</v>
+        <v>0.3287109070503538</v>
       </c>
       <c r="K14">
-        <v>0.7166666666666667</v>
+        <v>0.15</v>
       </c>
       <c r="L14">
         <v>0.8465119973270001</v>
@@ -1621,13 +1621,13 @@
         <v>0.5105365248548974</v>
       </c>
       <c r="R14">
-        <v>0.526472740859827</v>
+        <v>0.4165166364897969</v>
       </c>
       <c r="S14">
-        <v>0.5695706139311104</v>
+        <v>0.4658670209440876</v>
       </c>
       <c r="T14">
-        <v>0.999999999999999</v>
+        <v>0.05349551449880097</v>
       </c>
     </row>
     <row r="15" spans="1:20">
@@ -1635,7 +1635,7 @@
         <v>33</v>
       </c>
       <c r="B15">
-        <v>0.07832465980502792</v>
+        <v>0.07776726825200539</v>
       </c>
       <c r="C15" t="s">
         <v>134</v>
@@ -1671,7 +1671,7 @@
         <v>0.05</v>
       </c>
       <c r="N15">
-        <v>0.1574630820862223</v>
+        <v>0.0953901871284271</v>
       </c>
       <c r="O15">
         <v>0</v>
@@ -1680,13 +1680,13 @@
         <v>0.15</v>
       </c>
       <c r="Q15">
-        <v>0.08586155958038134</v>
+        <v>0.06994218440934979</v>
       </c>
       <c r="R15">
-        <v>0.102208619036763</v>
+        <v>0.09918202108109829</v>
       </c>
       <c r="S15">
-        <v>0.04590828305648947</v>
+        <v>0.0447934999504444</v>
       </c>
       <c r="T15">
         <v>0.1249239775786869</v>
@@ -1697,7 +1697,7 @@
         <v>34</v>
       </c>
       <c r="B16">
-        <v>0.04127969525862004</v>
+        <v>0.01638332391362192</v>
       </c>
       <c r="C16" t="s">
         <v>134</v>
@@ -1709,10 +1709,10 @@
         <v>0.01199770569238325</v>
       </c>
       <c r="F16">
-        <v>0.15</v>
+        <v>0</v>
       </c>
       <c r="G16">
-        <v>0.06822959303015641</v>
+        <v>0.021255721761705</v>
       </c>
       <c r="H16">
         <v>0.025</v>
@@ -1733,7 +1733,7 @@
         <v>0.01686125637994725</v>
       </c>
       <c r="N16">
-        <v>0.09090586453500203</v>
+        <v>0.01612693471314535</v>
       </c>
       <c r="O16">
         <v>0</v>
@@ -1742,16 +1742,16 @@
         <v>0</v>
       </c>
       <c r="Q16">
-        <v>0.04803529167817683</v>
+        <v>0.007781118938087882</v>
       </c>
       <c r="R16">
-        <v>0.0164741121635615</v>
+        <v>0.008820972790112666</v>
       </c>
       <c r="S16">
-        <v>0.01432979748708367</v>
+        <v>0.01151092606553884</v>
       </c>
       <c r="T16">
-        <v>0.2088148086683153</v>
+        <v>0.0416413258595623</v>
       </c>
     </row>
     <row r="17" spans="1:20">
@@ -1821,22 +1821,22 @@
         <v>36</v>
       </c>
       <c r="B18">
-        <v>0.1799622434537176</v>
+        <v>0.1486816565477629</v>
       </c>
       <c r="C18" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="D18">
-        <v>0.3444444444444444</v>
+        <v>0.2666666666666667</v>
       </c>
       <c r="E18">
-        <v>0.05698910203882045</v>
+        <v>0</v>
       </c>
       <c r="F18">
         <v>0</v>
       </c>
       <c r="G18">
-        <v>0.1375915225636771</v>
+        <v>0.09132927383832534</v>
       </c>
       <c r="H18">
         <v>0.3625</v>
@@ -1845,10 +1845,10 @@
         <v>0.1062220677453127</v>
       </c>
       <c r="J18">
-        <v>0.09836109573391963</v>
+        <v>0</v>
       </c>
       <c r="K18">
-        <v>0.1500000000000001</v>
+        <v>0</v>
       </c>
       <c r="L18">
         <v>0.234746357014</v>
@@ -1857,7 +1857,7 @@
         <v>0</v>
       </c>
       <c r="N18">
-        <v>0.1941197245235146</v>
+        <v>0.1236774504702864</v>
       </c>
       <c r="O18">
         <v>0.2916666666666666</v>
@@ -1866,16 +1866,16 @@
         <v>0.3625</v>
       </c>
       <c r="Q18">
-        <v>0.04978444657508348</v>
+        <v>0.03171863879672184</v>
       </c>
       <c r="R18">
-        <v>0.1915184419021119</v>
+        <v>0.1472674184707322</v>
       </c>
       <c r="S18">
-        <v>0.222332964343758</v>
+        <v>0.2060340392572005</v>
       </c>
       <c r="T18">
-        <v>0.2352584762324639</v>
+        <v>0.05349551449880097</v>
       </c>
     </row>
     <row r="19" spans="1:20">
@@ -1883,7 +1883,7 @@
         <v>37</v>
       </c>
       <c r="B19">
-        <v>0.3771684595563897</v>
+        <v>0.3225883696781638</v>
       </c>
       <c r="C19" t="s">
         <v>135</v>
@@ -1892,19 +1892,19 @@
         <v>0.2666666666666667</v>
       </c>
       <c r="E19">
-        <v>0.5693633348838272</v>
+        <v>0.380399470228791</v>
       </c>
       <c r="F19">
         <v>0.5</v>
       </c>
       <c r="G19">
-        <v>0.4439725715791108</v>
+        <v>0.3789017156360616</v>
       </c>
       <c r="H19">
-        <v>0.8087500000000001</v>
+        <v>0.72375</v>
       </c>
       <c r="I19">
-        <v>0.09526735953309873</v>
+        <v>0.04776365656895205</v>
       </c>
       <c r="J19">
         <v>0.07511013136381994</v>
@@ -1919,7 +1919,7 @@
         <v>0.1674183496349445</v>
       </c>
       <c r="N19">
-        <v>0.1957747106841858</v>
+        <v>0.1016191958605639</v>
       </c>
       <c r="O19">
         <v>0</v>
@@ -1928,16 +1928,16 @@
         <v>0</v>
       </c>
       <c r="Q19">
-        <v>0.1320673979057297</v>
+        <v>0.1079200310732661</v>
       </c>
       <c r="R19">
-        <v>0.03908893709057132</v>
+        <v>0.03449803007916986</v>
       </c>
       <c r="S19">
-        <v>0.3103643475336685</v>
+        <v>0.266275023720266</v>
       </c>
       <c r="T19">
-        <v>0.971580507922511</v>
+        <v>0.886322031690047</v>
       </c>
     </row>
     <row r="20" spans="1:20">
@@ -1945,10 +1945,10 @@
         <v>38</v>
       </c>
       <c r="B20">
-        <v>0.1552544321734411</v>
+        <v>0.1065343698353132</v>
       </c>
       <c r="C20" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="D20">
         <v>0.15</v>
@@ -1966,7 +1966,7 @@
         <v>0.15</v>
       </c>
       <c r="I20">
-        <v>0.3174270899922695</v>
+        <v>0</v>
       </c>
       <c r="J20">
         <v>0.1500000000000001</v>
@@ -1981,7 +1981,7 @@
         <v>0.06962306263125041</v>
       </c>
       <c r="N20">
-        <v>0.2720604843770376</v>
+        <v>0.1700127676436622</v>
       </c>
       <c r="O20">
         <v>0.15</v>
@@ -1990,16 +1990,16 @@
         <v>0.15</v>
       </c>
       <c r="Q20">
-        <v>0.1405699074896956</v>
+        <v>0.1143984861449957</v>
       </c>
       <c r="R20">
-        <v>0.1482071470512861</v>
+        <v>0.1432314259888887</v>
       </c>
       <c r="S20">
-        <v>0.1997678277933157</v>
+        <v>0.10232770311706</v>
       </c>
       <c r="T20">
-        <v>0.1499999999999999</v>
+        <v>0.02507602242131295</v>
       </c>
     </row>
     <row r="21" spans="1:20">
@@ -2007,7 +2007,7 @@
         <v>39</v>
       </c>
       <c r="B21">
-        <v>0.1349962317563093</v>
+        <v>0.1287789687008479</v>
       </c>
       <c r="C21" t="s">
         <v>134</v>
@@ -2031,7 +2031,7 @@
         <v>0.07925143034772975</v>
       </c>
       <c r="J21">
-        <v>0.5070409081456229</v>
+        <v>0.3381681332445731</v>
       </c>
       <c r="K21">
         <v>0.15</v>
@@ -2043,7 +2043,7 @@
         <v>0.1861247399954011</v>
       </c>
       <c r="N21">
-        <v>0.2215890752986185</v>
+        <v>0.1738630250995395</v>
       </c>
       <c r="O21">
         <v>1</v>
@@ -2052,13 +2052,13 @@
         <v>0.15</v>
       </c>
       <c r="Q21">
-        <v>0.3085298203763837</v>
+        <v>0.2962898741153431</v>
       </c>
       <c r="R21">
-        <v>0.3779059929339446</v>
+        <v>0.3441466803798701</v>
       </c>
       <c r="S21">
-        <v>0.179587593357992</v>
+        <v>0.1671530672470693</v>
       </c>
       <c r="T21">
         <v>0</v>
@@ -2069,7 +2069,7 @@
         <v>40</v>
       </c>
       <c r="B22">
-        <v>0.2516855283637547</v>
+        <v>0.1701624630940777</v>
       </c>
       <c r="C22" t="s">
         <v>135</v>
@@ -2087,13 +2087,13 @@
         <v>0.2504524566717806</v>
       </c>
       <c r="H22">
-        <v>0.3425</v>
+        <v>0.07500000000000001</v>
       </c>
       <c r="I22">
         <v>0.05845841117636069</v>
       </c>
       <c r="J22">
-        <v>0.4960620457289249</v>
+        <v>0</v>
       </c>
       <c r="K22">
         <v>0</v>
@@ -2102,28 +2102,28 @@
         <v>0.54172236234</v>
       </c>
       <c r="M22">
-        <v>0.5194001913586258</v>
+        <v>0.2527280111046633</v>
       </c>
       <c r="N22">
-        <v>0.5938153397785682</v>
+        <v>0.1928494253165867</v>
       </c>
       <c r="O22">
-        <v>0.3250000000000001</v>
+        <v>0</v>
       </c>
       <c r="P22">
         <v>0.15</v>
       </c>
       <c r="Q22">
-        <v>0.4273216725550035</v>
+        <v>0.1111202516243557</v>
       </c>
       <c r="R22">
-        <v>0.3315599926192839</v>
+        <v>0.1289048627352814</v>
       </c>
       <c r="S22">
-        <v>0.2529186000557288</v>
+        <v>0.08987246951637487</v>
       </c>
       <c r="T22">
-        <v>0.1734042875932253</v>
+        <v>0.1617021437966126</v>
       </c>
     </row>
     <row r="23" spans="1:20">
@@ -2131,7 +2131,7 @@
         <v>41</v>
       </c>
       <c r="B23">
-        <v>0.2447682063683087</v>
+        <v>0.2071100381924364</v>
       </c>
       <c r="C23" t="s">
         <v>135</v>
@@ -2140,22 +2140,22 @@
         <v>0.05</v>
       </c>
       <c r="E23">
-        <v>0.4373885722676115</v>
+        <v>0.380399470228791</v>
       </c>
       <c r="F23">
         <v>0.5</v>
       </c>
       <c r="G23">
-        <v>0.3243212244982625</v>
+        <v>0.3046966806424223</v>
       </c>
       <c r="H23">
-        <v>0.135</v>
+        <v>0.025</v>
       </c>
       <c r="I23">
-        <v>0.1665993756029285</v>
+        <v>0.1215439275378373</v>
       </c>
       <c r="J23">
-        <v>0.2880827722160289</v>
+        <v>0.2066895463276636</v>
       </c>
       <c r="K23">
         <v>0.15</v>
@@ -2167,7 +2167,7 @@
         <v>0.2412848783867689</v>
       </c>
       <c r="N23">
-        <v>0.2367990352443523</v>
+        <v>0.2262833023209607</v>
       </c>
       <c r="O23">
         <v>0.2083333333333333</v>
@@ -2176,16 +2176,16 @@
         <v>0.15</v>
       </c>
       <c r="Q23">
-        <v>0.1701137881435582</v>
+        <v>0.1674168960827052</v>
       </c>
       <c r="R23">
-        <v>0.1911933218326338</v>
+        <v>0.1755308860252745</v>
       </c>
       <c r="S23">
-        <v>0.165215188238355</v>
+        <v>0.1095233957424505</v>
       </c>
       <c r="T23">
-        <v>0.2920974603874399</v>
+        <v>0</v>
       </c>
     </row>
     <row r="24" spans="1:20">
@@ -2193,7 +2193,7 @@
         <v>42</v>
       </c>
       <c r="B24">
-        <v>0.0795924348345935</v>
+        <v>0.0680257636393225</v>
       </c>
       <c r="C24" t="s">
         <v>134</v>
@@ -2211,7 +2211,7 @@
         <v>0.021255721761705</v>
       </c>
       <c r="H24">
-        <v>0.325</v>
+        <v>0.255</v>
       </c>
       <c r="I24">
         <v>0.02079301917136905</v>
@@ -2244,7 +2244,7 @@
         <v>0.06586939259395025</v>
       </c>
       <c r="S24">
-        <v>0.137929147907482</v>
+        <v>0.11479580551694</v>
       </c>
       <c r="T24">
         <v>0.1499999999999999</v>
@@ -2255,7 +2255,7 @@
         <v>43</v>
       </c>
       <c r="B25">
-        <v>0.04631537313536227</v>
+        <v>0.03670459601424927</v>
       </c>
       <c r="C25" t="s">
         <v>134</v>
@@ -2279,7 +2279,7 @@
         <v>0</v>
       </c>
       <c r="J25">
-        <v>0.31651722992113</v>
+        <v>0.07478904058924606</v>
       </c>
       <c r="K25">
         <v>0</v>
@@ -2291,7 +2291,7 @@
         <v>0.4984703064604985</v>
       </c>
       <c r="N25">
-        <v>0.3632591556493465</v>
+        <v>0.215735915815121</v>
       </c>
       <c r="O25">
         <v>0.5</v>
@@ -2300,16 +2300,16 @@
         <v>0</v>
       </c>
       <c r="Q25">
-        <v>0.2124808595000839</v>
+        <v>0.1746466678941682</v>
       </c>
       <c r="R25">
-        <v>0.1841969120484387</v>
+        <v>0.1320110505487877</v>
       </c>
       <c r="S25">
-        <v>0.09263074627072454</v>
+        <v>0.07340919202849853</v>
       </c>
       <c r="T25">
-        <v>0.110334498653777</v>
+        <v>0.02507602242131295</v>
       </c>
     </row>
     <row r="26" spans="1:20">
@@ -2317,13 +2317,13 @@
         <v>44</v>
       </c>
       <c r="B26">
-        <v>0.5761212727234799</v>
+        <v>0.4574570081257169</v>
       </c>
       <c r="C26" t="s">
         <v>136</v>
       </c>
       <c r="D26">
-        <v>1</v>
+        <v>0.5277777777777778</v>
       </c>
       <c r="E26">
         <v>0.8170349881911554</v>
@@ -2332,13 +2332,13 @@
         <v>0.2714285714285715</v>
       </c>
       <c r="G26">
-        <v>0.7088360822115525</v>
+        <v>0.5471071597895181</v>
       </c>
       <c r="H26">
         <v>0.4475</v>
       </c>
       <c r="I26">
-        <v>0.2779695903699899</v>
+        <v>0.026970637397583</v>
       </c>
       <c r="J26">
         <v>0.5704367083174489</v>
@@ -2368,10 +2368,10 @@
         <v>0.5750169446062644</v>
       </c>
       <c r="S26">
-        <v>0.4434064632354073</v>
+        <v>0.3678068564619156</v>
       </c>
       <c r="T26">
-        <v>0.1617021437966126</v>
+        <v>0.1249239775786869</v>
       </c>
     </row>
     <row r="27" spans="1:20">
@@ -2441,13 +2441,13 @@
         <v>46</v>
       </c>
       <c r="B28">
-        <v>0.2622948860910188</v>
+        <v>0.0848889868469461</v>
       </c>
       <c r="C28" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="D28">
-        <v>0.6222222222222222</v>
+        <v>0</v>
       </c>
       <c r="E28">
         <v>0</v>
@@ -2456,19 +2456,19 @@
         <v>0.05</v>
       </c>
       <c r="G28">
-        <v>0.2287595960455762</v>
+        <v>0.0156579570894838</v>
       </c>
       <c r="H28">
-        <v>0.6799999999999999</v>
+        <v>0.2875</v>
       </c>
       <c r="I28">
         <v>0.07235849582160145</v>
       </c>
       <c r="J28">
-        <v>0.08699278091547852</v>
+        <v>0.05154648835437114</v>
       </c>
       <c r="K28">
-        <v>0.1500000000000001</v>
+        <v>0</v>
       </c>
       <c r="L28">
         <v>0</v>
@@ -2477,7 +2477,7 @@
         <v>0.5931576716389991</v>
       </c>
       <c r="N28">
-        <v>0.4366514549540532</v>
+        <v>0.3655117326428723</v>
       </c>
       <c r="O28">
         <v>0.2666666666666667</v>
@@ -2486,16 +2486,16 @@
         <v>0.05</v>
       </c>
       <c r="Q28">
-        <v>0.2402170044754073</v>
+        <v>0.2219723273131015</v>
       </c>
       <c r="R28">
-        <v>0.1338811190491588</v>
+        <v>0.1013064061242945</v>
       </c>
       <c r="S28">
-        <v>0.2958301761364613</v>
+        <v>0.1541200166044084</v>
       </c>
       <c r="T28">
-        <v>0.999999999999999</v>
+        <v>0.8579025396125589</v>
       </c>
     </row>
     <row r="29" spans="1:20">
@@ -2503,7 +2503,7 @@
         <v>47</v>
       </c>
       <c r="B29">
-        <v>0.1397893153409261</v>
+        <v>0.06974820787170899</v>
       </c>
       <c r="C29" t="s">
         <v>134</v>
@@ -2521,16 +2521,16 @@
         <v>0</v>
       </c>
       <c r="H29">
-        <v>0.5962500000000001</v>
+        <v>0.3412500000000001</v>
       </c>
       <c r="I29">
         <v>0.02429690983669855</v>
       </c>
       <c r="J29">
-        <v>0.2760732839236957</v>
+        <v>0.03976466684964675</v>
       </c>
       <c r="K29">
-        <v>0.7166666666666667</v>
+        <v>0</v>
       </c>
       <c r="L29">
         <v>0.0687416456475</v>
@@ -2551,10 +2551,10 @@
         <v>0.06098424390713934</v>
       </c>
       <c r="R29">
-        <v>0.2042034869137338</v>
+        <v>0.05267920282069909</v>
       </c>
       <c r="S29">
-        <v>0.2795786306818522</v>
+        <v>0.139496415743418</v>
       </c>
       <c r="T29">
         <v>0.04999999999999995</v>
@@ -2565,7 +2565,7 @@
         <v>48</v>
       </c>
       <c r="B30">
-        <v>0.2500196458293833</v>
+        <v>0.2421484872653828</v>
       </c>
       <c r="C30" t="s">
         <v>135</v>
@@ -2583,13 +2583,13 @@
         <v>0.2556250841747643</v>
       </c>
       <c r="H30">
-        <v>0.42125</v>
+        <v>0.38625</v>
       </c>
       <c r="I30">
         <v>0.09051649050796064</v>
       </c>
       <c r="J30">
-        <v>0.2248395012468233</v>
+        <v>0.187725812187153</v>
       </c>
       <c r="K30">
         <v>0.05</v>
@@ -2601,7 +2601,7 @@
         <v>0.5182267485159716</v>
       </c>
       <c r="N30">
-        <v>0.3364274883402757</v>
+        <v>0.2455971876441166</v>
       </c>
       <c r="O30">
         <v>0.2083333333333333</v>
@@ -2610,16 +2610,16 @@
         <v>0.2375</v>
       </c>
       <c r="Q30">
-        <v>0.2540593653522476</v>
+        <v>0.2307647915344337</v>
       </c>
       <c r="R30">
-        <v>0.2115988695821441</v>
+        <v>0.2002621338753967</v>
       </c>
       <c r="S30">
-        <v>0.2444142074840023</v>
+        <v>0.2286718903560013</v>
       </c>
       <c r="T30">
-        <v>0.4765957124067741</v>
+        <v>0.4648935686101614</v>
       </c>
     </row>
     <row r="31" spans="1:20">
@@ -2627,7 +2627,7 @@
         <v>49</v>
       </c>
       <c r="B31">
-        <v>0.2566460693688007</v>
+        <v>0.1585823941813442</v>
       </c>
       <c r="C31" t="s">
         <v>135</v>
@@ -2645,43 +2645,43 @@
         <v>0.0469738712684514</v>
       </c>
       <c r="H31">
-        <v>1</v>
+        <v>0.72375</v>
       </c>
       <c r="I31">
-        <v>0.1262655401831711</v>
+        <v>0</v>
       </c>
       <c r="J31">
-        <v>0.2712235801380304</v>
+        <v>0.0583215113794819</v>
       </c>
       <c r="K31">
         <v>0</v>
       </c>
       <c r="L31">
-        <v>0.190099293292875</v>
+        <v>0.081258354351</v>
       </c>
       <c r="M31">
         <v>0.7159379044644983</v>
       </c>
       <c r="N31">
-        <v>0.2518787389164502</v>
+        <v>0.1704059961255277</v>
       </c>
       <c r="O31">
-        <v>0.3250000000000001</v>
+        <v>0.1500000000000001</v>
       </c>
       <c r="P31">
-        <v>0.325</v>
+        <v>0</v>
       </c>
       <c r="Q31">
-        <v>0.4299833880246933</v>
+        <v>0.1984783437150242</v>
       </c>
       <c r="R31">
-        <v>0.2655546277392991</v>
+        <v>0.0841875058733528</v>
       </c>
       <c r="S31">
-        <v>0.4663182674691501</v>
+        <v>0.270190917094237</v>
       </c>
       <c r="T31">
-        <v>0.999999999999999</v>
+        <v>0.05349551449880097</v>
       </c>
     </row>
     <row r="32" spans="1:20">
@@ -2689,7 +2689,7 @@
         <v>50</v>
       </c>
       <c r="B32">
-        <v>0.0003593598012469021</v>
+        <v>0.000245018046304706</v>
       </c>
       <c r="C32" t="s">
         <v>134</v>
@@ -2725,7 +2725,7 @@
         <v>0</v>
       </c>
       <c r="N32">
-        <v>0.04001944965597876</v>
+        <v>0.02728598840180371</v>
       </c>
       <c r="O32">
         <v>0</v>
@@ -2734,16 +2734,16 @@
         <v>0</v>
       </c>
       <c r="Q32">
-        <v>0.01026349155529003</v>
+        <v>0.00699783515133411</v>
       </c>
       <c r="R32">
-        <v>0.001951299107250669</v>
+        <v>0.001330431209489092</v>
       </c>
       <c r="S32">
-        <v>0.0007187196024938042</v>
+        <v>0.000490036092609412</v>
       </c>
       <c r="T32">
-        <v>0.999999999999999</v>
+        <v>0.7684437828976594</v>
       </c>
     </row>
     <row r="33" spans="1:20">
@@ -2867,7 +2867,7 @@
         <v>0.05002296119533625</v>
       </c>
       <c r="T34">
-        <v>0.8930089710023971</v>
+        <v>0.8696046834091716</v>
       </c>
     </row>
     <row r="35" spans="1:20">
@@ -2937,7 +2937,7 @@
         <v>54</v>
       </c>
       <c r="B36">
-        <v>0.5571659207979689</v>
+        <v>0.5313242153809947</v>
       </c>
       <c r="C36" t="s">
         <v>136</v>
@@ -2958,13 +2958,13 @@
         <v>1</v>
       </c>
       <c r="I36">
-        <v>0.29258419316408</v>
+        <v>0.2238153513805199</v>
       </c>
       <c r="J36">
-        <v>0.3521539754597796</v>
+        <v>0.2497535747276917</v>
       </c>
       <c r="K36">
-        <v>0.4333333333333333</v>
+        <v>0</v>
       </c>
       <c r="L36">
         <v>0.7291388188200001</v>
@@ -2985,13 +2985,13 @@
         <v>0.7011785593004816</v>
       </c>
       <c r="R36">
-        <v>0.532912530572704</v>
+        <v>0.4488284507603281</v>
       </c>
       <c r="S36">
-        <v>0.6148882068331445</v>
+        <v>0.5632047959991962</v>
       </c>
       <c r="T36">
-        <v>0.999999999999999</v>
+        <v>0.971580507922511</v>
       </c>
     </row>
     <row r="37" spans="1:20">
@@ -2999,7 +2999,7 @@
         <v>55</v>
       </c>
       <c r="B37">
-        <v>0.167478177615613</v>
+        <v>0.1610471378321647</v>
       </c>
       <c r="C37" t="s">
         <v>135</v>
@@ -3020,7 +3020,7 @@
         <v>0.15</v>
       </c>
       <c r="I37">
-        <v>0.04270350921283976</v>
+        <v>0</v>
       </c>
       <c r="J37">
         <v>0.07079175707528054</v>
@@ -3050,7 +3050,7 @@
         <v>0.1172413679059125</v>
       </c>
       <c r="S37">
-        <v>0.1056168965258184</v>
+        <v>0.09275481695892171</v>
       </c>
       <c r="T37">
         <v>0.1499999999999999</v>
@@ -3061,7 +3061,7 @@
         <v>56</v>
       </c>
       <c r="B38">
-        <v>0.02658883613440775</v>
+        <v>0.017062113299654</v>
       </c>
       <c r="C38" t="s">
         <v>134</v>
@@ -3085,10 +3085,10 @@
         <v>0.0300023387141979</v>
       </c>
       <c r="J38">
-        <v>0.1380473407692843</v>
+        <v>0.07511013136381997</v>
       </c>
       <c r="K38">
-        <v>0.2666666666666667</v>
+        <v>0</v>
       </c>
       <c r="L38">
         <v>0.108840938941875</v>
@@ -3109,10 +3109,10 @@
         <v>0.07530506887485158</v>
       </c>
       <c r="R38">
-        <v>0.1198416307382661</v>
+        <v>0.06811217825644154</v>
       </c>
       <c r="S38">
-        <v>0.0531776722688155</v>
+        <v>0.034124226599308</v>
       </c>
       <c r="T38">
         <v>0.1249239775786869</v>
@@ -3185,13 +3185,13 @@
         <v>58</v>
       </c>
       <c r="B40">
-        <v>0.3057862994543519</v>
+        <v>0.2779276928994642</v>
       </c>
       <c r="C40" t="s">
         <v>135</v>
       </c>
       <c r="D40">
-        <v>0.2277777777777778</v>
+        <v>0.1888888888888889</v>
       </c>
       <c r="E40">
         <v>0.03599311707714975</v>
@@ -3200,13 +3200,13 @@
         <v>0.25</v>
       </c>
       <c r="G40">
-        <v>0.1686946556020456</v>
+        <v>0.1553758031672898</v>
       </c>
       <c r="H40">
-        <v>1</v>
+        <v>0.915</v>
       </c>
       <c r="I40">
-        <v>0.1206914613030444</v>
+        <v>0.07318775833889768</v>
       </c>
       <c r="J40">
         <v>0.2509993391096323</v>
@@ -3236,10 +3236,10 @@
         <v>0.20647306343793</v>
       </c>
       <c r="S40">
-        <v>0.4428779433066581</v>
+        <v>0.4004795826316385</v>
       </c>
       <c r="T40">
-        <v>0.2920974603874399</v>
+        <v>0.1784194920774879</v>
       </c>
     </row>
     <row r="41" spans="1:20">
@@ -3247,13 +3247,13 @@
         <v>59</v>
       </c>
       <c r="B41">
-        <v>0.2960829195923323</v>
+        <v>0.2684905466777674</v>
       </c>
       <c r="C41" t="s">
         <v>135</v>
       </c>
       <c r="D41">
-        <v>0.8111111111111111</v>
+        <v>0.7166666666666667</v>
       </c>
       <c r="E41">
         <v>0</v>
@@ -3262,7 +3262,7 @@
         <v>0.2000000000000001</v>
       </c>
       <c r="G41">
-        <v>0.3404250362828414</v>
+        <v>0.3080792517984345</v>
       </c>
       <c r="H41">
         <v>0.5325</v>
@@ -3271,10 +3271,10 @@
         <v>0.09255915102923779</v>
       </c>
       <c r="J41">
-        <v>0.2215374065497922</v>
+        <v>0.1033830980127677</v>
       </c>
       <c r="K41">
-        <v>0.2666666666666667</v>
+        <v>0</v>
       </c>
       <c r="L41">
         <v>0</v>
@@ -3295,10 +3295,10 @@
         <v>0.04868486970603911</v>
       </c>
       <c r="R41">
-        <v>0.1300029246994121</v>
+        <v>0.06799592679945608</v>
       </c>
       <c r="S41">
-        <v>0.2517408029018233</v>
+        <v>0.2289018415571002</v>
       </c>
       <c r="T41">
         <v>0.999999999999999</v>
@@ -3309,13 +3309,13 @@
         <v>60</v>
       </c>
       <c r="B42">
-        <v>0.685307919248517</v>
+        <v>0.581540638089145</v>
       </c>
       <c r="C42" t="s">
         <v>136</v>
       </c>
       <c r="D42">
-        <v>0.9055555555555556</v>
+        <v>0.7166666666666667</v>
       </c>
       <c r="E42">
         <v>0.239954113847665</v>
@@ -3324,19 +3324,19 @@
         <v>0.7571428571428571</v>
       </c>
       <c r="G42">
-        <v>0.6298748581047334</v>
+        <v>0.5651832891359196</v>
       </c>
       <c r="H42">
         <v>1</v>
       </c>
       <c r="I42">
-        <v>0.4082672790557718</v>
+        <v>0.1636053420221653</v>
       </c>
       <c r="J42">
-        <v>0.9549333775704013</v>
+        <v>0.5400308276798762</v>
       </c>
       <c r="K42">
-        <v>0.7166666666666667</v>
+        <v>0</v>
       </c>
       <c r="L42">
         <v>0.45827763765</v>
@@ -3345,7 +3345,7 @@
         <v>0.6714158282289471</v>
       </c>
       <c r="N42">
-        <v>0.6982892840813785</v>
+        <v>0.637181214397551</v>
       </c>
       <c r="O42">
         <v>1</v>
@@ -3354,16 +3354,16 @@
         <v>0.7875</v>
       </c>
       <c r="Q42">
-        <v>0.7321556116679401</v>
+        <v>0.7164836780818584</v>
       </c>
       <c r="R42">
-        <v>0.7800005240982092</v>
+        <v>0.5922550398610107</v>
       </c>
       <c r="S42">
-        <v>0.7407409803923006</v>
+        <v>0.5978979870423703</v>
       </c>
       <c r="T42">
-        <v>0.999999999999999</v>
+        <v>0.6833320271370084</v>
       </c>
     </row>
     <row r="43" spans="1:20">
@@ -3371,10 +3371,10 @@
         <v>61</v>
       </c>
       <c r="B43">
-        <v>0.7140964771925215</v>
+        <v>0.6543414040551794</v>
       </c>
       <c r="C43" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="D43">
         <v>0.9055555555555556</v>
@@ -3389,16 +3389,16 @@
         <v>0.8366613446126938</v>
       </c>
       <c r="H43">
-        <v>1</v>
+        <v>0.915</v>
       </c>
       <c r="I43">
-        <v>0.2309726832865759</v>
+        <v>0.0693100639045635</v>
       </c>
       <c r="J43">
-        <v>0.6639005984831369</v>
+        <v>0.3532844720367061</v>
       </c>
       <c r="K43">
-        <v>0.2666666666666667</v>
+        <v>0</v>
       </c>
       <c r="L43">
         <v>0.35660047113325</v>
@@ -3407,7 +3407,7 @@
         <v>0.7881448157309003</v>
       </c>
       <c r="N43">
-        <v>0.7980586243433435</v>
+        <v>0.4253179703591951</v>
       </c>
       <c r="O43">
         <v>0.2666666666666667</v>
@@ -3416,16 +3416,16 @@
         <v>1</v>
       </c>
       <c r="Q43">
-        <v>0.4958388234346103</v>
+        <v>0.4002447913485631</v>
       </c>
       <c r="R43">
-        <v>0.5198819873975027</v>
+        <v>0.4038777419898558</v>
       </c>
       <c r="S43">
-        <v>0.5915316097723491</v>
+        <v>0.4720214634976649</v>
       </c>
       <c r="T43">
-        <v>0.7685905033694724</v>
+        <v>0.4952341854122916</v>
       </c>
     </row>
     <row r="44" spans="1:20">
@@ -3433,61 +3433,61 @@
         <v>62</v>
       </c>
       <c r="B44">
-        <v>0.253503310132717</v>
+        <v>0.1085588359929428</v>
       </c>
       <c r="C44" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="D44">
-        <v>0.3055555555555556</v>
+        <v>0.2666666666666667</v>
       </c>
       <c r="E44">
-        <v>0.05698910203882045</v>
+        <v>0</v>
       </c>
       <c r="F44">
         <v>0.15</v>
       </c>
       <c r="G44">
-        <v>0.1712465413973727</v>
+        <v>0.1383031451067767</v>
       </c>
       <c r="H44">
-        <v>0.45125</v>
+        <v>0</v>
       </c>
       <c r="I44">
         <v>0.0284560724621628</v>
       </c>
       <c r="J44">
-        <v>0.6272569008377629</v>
+        <v>0.1652433762230192</v>
       </c>
       <c r="K44">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L44">
-        <v>0.2132009422715</v>
+        <v>0.0687416456475</v>
       </c>
       <c r="M44">
         <v>0.3507359301054291</v>
       </c>
       <c r="N44">
-        <v>0.4812994510853836</v>
+        <v>0.2208734631805265</v>
       </c>
       <c r="O44">
-        <v>0.4333333333333333</v>
+        <v>0.2916666666666666</v>
       </c>
       <c r="P44">
         <v>0.4125</v>
       </c>
       <c r="Q44">
-        <v>0.2550044734127387</v>
+        <v>0.1882149510525719</v>
       </c>
       <c r="R44">
-        <v>0.483431730780037</v>
+        <v>0.1907092473118617</v>
       </c>
       <c r="S44">
-        <v>0.3357600788680613</v>
+        <v>0.07881452687910882</v>
       </c>
       <c r="T44">
-        <v>0.943161015845023</v>
+        <v>0.8579025396125589</v>
       </c>
     </row>
     <row r="45" spans="1:20">
@@ -3495,10 +3495,10 @@
         <v>63</v>
       </c>
       <c r="B45">
-        <v>0.1843937249378793</v>
+        <v>0.1319460747475913</v>
       </c>
       <c r="C45" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="D45">
         <v>0.2277777777777778</v>
@@ -3507,16 +3507,16 @@
         <v>0.05698910203882045</v>
       </c>
       <c r="F45">
-        <v>0.2000000000000001</v>
+        <v>0</v>
       </c>
       <c r="G45">
-        <v>0.160266793617345</v>
+        <v>0.0976349652594098</v>
       </c>
       <c r="H45">
         <v>0.3412500000000001</v>
       </c>
       <c r="I45">
-        <v>0.1888064142589102</v>
+        <v>0.08210004905292449</v>
       </c>
       <c r="J45">
         <v>0.03976466684964675</v>
@@ -3525,13 +3525,13 @@
         <v>0</v>
       </c>
       <c r="L45">
-        <v>0.2132009422715</v>
+        <v>0.0687416456475</v>
       </c>
       <c r="M45">
-        <v>0.09489999717557235</v>
+        <v>0.01686125637994725</v>
       </c>
       <c r="N45">
-        <v>0.1423659146213465</v>
+        <v>0.09744727913986034</v>
       </c>
       <c r="O45">
         <v>0.15</v>
@@ -3540,16 +3540,16 @@
         <v>0.15</v>
       </c>
       <c r="Q45">
-        <v>0.09169644106131353</v>
+        <v>0.06330562701316345</v>
       </c>
       <c r="R45">
-        <v>0.1055526594679109</v>
+        <v>0.07806618850407826</v>
       </c>
       <c r="S45">
-        <v>0.2085206562584136</v>
+        <v>0.1662571842357729</v>
       </c>
       <c r="T45">
-        <v>0.2085107189830634</v>
+        <v>0.1249239775786869</v>
       </c>
     </row>
     <row r="46" spans="1:20">
@@ -3557,13 +3557,13 @@
         <v>64</v>
       </c>
       <c r="B46">
-        <v>0.1151510632441528</v>
+        <v>0.1241740559446883</v>
       </c>
       <c r="C46" t="s">
         <v>134</v>
       </c>
       <c r="D46">
-        <v>0.2666666666666667</v>
+        <v>0.2277777777777778</v>
       </c>
       <c r="E46">
         <v>0</v>
@@ -3572,19 +3572,19 @@
         <v>0.2000000000000001</v>
       </c>
       <c r="G46">
-        <v>0.1539611021962606</v>
+        <v>0.1406422497615048</v>
       </c>
       <c r="H46">
-        <v>0.11</v>
+        <v>0.245</v>
       </c>
       <c r="I46">
         <v>0</v>
       </c>
       <c r="J46">
-        <v>0.1787645381196142</v>
+        <v>0.1157489068998678</v>
       </c>
       <c r="K46">
-        <v>0.1500000000000001</v>
+        <v>0</v>
       </c>
       <c r="L46">
         <v>0</v>
@@ -3593,7 +3593,7 @@
         <v>0.4622663138922483</v>
       </c>
       <c r="N46">
-        <v>0.3639721330864938</v>
+        <v>0.3284022719309033</v>
       </c>
       <c r="O46">
         <v>0.05</v>
@@ -3602,16 +3602,16 @@
         <v>0.05</v>
       </c>
       <c r="Q46">
-        <v>0.1932806297464422</v>
+        <v>0.1841582911652893</v>
       </c>
       <c r="R46">
-        <v>0.1085677585608354</v>
+        <v>0.07259591389239892</v>
       </c>
       <c r="S46">
-        <v>0.07634102429204506</v>
+        <v>0.1077058621278718</v>
       </c>
       <c r="T46">
-        <v>0.2687509652236004</v>
+        <v>0.03677816621792566</v>
       </c>
     </row>
     <row r="47" spans="1:20">
@@ -3619,13 +3619,13 @@
         <v>65</v>
       </c>
       <c r="B47">
-        <v>0.2424840139543374</v>
+        <v>0.1919885091876309</v>
       </c>
       <c r="C47" t="s">
         <v>135</v>
       </c>
       <c r="D47">
-        <v>0.3055555555555556</v>
+        <v>0.2277777777777778</v>
       </c>
       <c r="E47">
         <v>0</v>
@@ -3634,16 +3634,16 @@
         <v>0.6357142857142857</v>
       </c>
       <c r="G47">
-        <v>0.3037278664108037</v>
+        <v>0.2770901615412922</v>
       </c>
       <c r="H47">
-        <v>0.38625</v>
+        <v>0.18</v>
       </c>
       <c r="I47">
         <v>0</v>
       </c>
       <c r="J47">
-        <v>0.204981833688714</v>
+        <v>0.1146545354858269</v>
       </c>
       <c r="K47">
         <v>0.15</v>
@@ -3667,10 +3667,10 @@
         <v>0.07252939825905463</v>
       </c>
       <c r="R47">
-        <v>0.1455050138216133</v>
+        <v>0.1286924154711384</v>
       </c>
       <c r="S47">
-        <v>0.1812401614978712</v>
+        <v>0.1068868568339697</v>
       </c>
       <c r="T47">
         <v>0.1499999999999999</v>
@@ -3681,7 +3681,7 @@
         <v>66</v>
       </c>
       <c r="B48">
-        <v>0.1244487292913076</v>
+        <v>0.05504138317634134</v>
       </c>
       <c r="C48" t="s">
         <v>134</v>
@@ -3699,7 +3699,7 @@
         <v>0.02685463896062348</v>
       </c>
       <c r="H48">
-        <v>0.5775</v>
+        <v>0.1625</v>
       </c>
       <c r="I48">
         <v>0.00693100639045635</v>
@@ -3717,7 +3717,7 @@
         <v>0</v>
       </c>
       <c r="N48">
-        <v>0.3862061289880359</v>
+        <v>0.293383834780083</v>
       </c>
       <c r="O48">
         <v>0</v>
@@ -3726,13 +3726,13 @@
         <v>0</v>
       </c>
       <c r="Q48">
-        <v>0.1337163048657043</v>
+        <v>0.109910859240251</v>
       </c>
       <c r="R48">
-        <v>0.07901951553707803</v>
+        <v>0.07449361472190083</v>
       </c>
       <c r="S48">
-        <v>0.2220428196219917</v>
+        <v>0.08322812739205919</v>
       </c>
       <c r="T48">
         <v>0.0835867414043765</v>
@@ -3743,7 +3743,7 @@
         <v>67</v>
       </c>
       <c r="B49">
-        <v>0.0981520402679246</v>
+        <v>0.05317345160449295</v>
       </c>
       <c r="C49" t="s">
         <v>134</v>
@@ -3764,7 +3764,7 @@
         <v>0.05</v>
       </c>
       <c r="I49">
-        <v>0.2949117333644151</v>
+        <v>0</v>
       </c>
       <c r="J49">
         <v>0.05000000000000005</v>
@@ -3779,7 +3779,7 @@
         <v>0.05</v>
       </c>
       <c r="N49">
-        <v>0.1510702461154928</v>
+        <v>0.08807963182747158</v>
       </c>
       <c r="O49">
         <v>0.2083333333333333</v>
@@ -3788,16 +3788,16 @@
         <v>0.325</v>
       </c>
       <c r="Q49">
-        <v>0.1333362861692876</v>
+        <v>0.1171815503254615</v>
       </c>
       <c r="R49">
-        <v>0.1579354112080131</v>
+        <v>0.1548640663873823</v>
       </c>
       <c r="S49">
-        <v>0.1635218846016794</v>
+        <v>0.07356470727481611</v>
       </c>
       <c r="T49">
-        <v>0.2068389841549759</v>
+        <v>0</v>
       </c>
     </row>
     <row r="50" spans="1:20">
@@ -3805,13 +3805,13 @@
         <v>68</v>
       </c>
       <c r="B50">
-        <v>0.1628307083765363</v>
+        <v>0.1226798944084742</v>
       </c>
       <c r="C50" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="D50">
-        <v>0.3444444444444444</v>
+        <v>0.1888888888888889</v>
       </c>
       <c r="E50">
         <v>0.07798508700049113</v>
@@ -3820,7 +3820,7 @@
         <v>0.15</v>
       </c>
       <c r="G50">
-        <v>0.1917954889369118</v>
+        <v>0.1385200791978887</v>
       </c>
       <c r="H50">
         <v>0.1</v>
@@ -3844,22 +3844,22 @@
         <v>0.111063973336967</v>
       </c>
       <c r="O50">
-        <v>0.575</v>
+        <v>0.2916666666666666</v>
       </c>
       <c r="P50">
         <v>0.2375</v>
       </c>
       <c r="Q50">
-        <v>0.2204793235904275</v>
+        <v>0.0647613864723145</v>
       </c>
       <c r="R50">
-        <v>0.2089116422464974</v>
+        <v>0.1355363853905807</v>
       </c>
       <c r="S50">
-        <v>0.1338659278161608</v>
+        <v>0.1068397096190597</v>
       </c>
       <c r="T50">
-        <v>0.999999999999999</v>
+        <v>0.167173482808753</v>
       </c>
     </row>
     <row r="51" spans="1:20">
@@ -3867,7 +3867,7 @@
         <v>69</v>
       </c>
       <c r="B51">
-        <v>0.5230686422686167</v>
+        <v>0.433717959769883</v>
       </c>
       <c r="C51" t="s">
         <v>136</v>
@@ -3879,19 +3879,19 @@
         <v>0.1199770569238325</v>
       </c>
       <c r="F51">
-        <v>0.4</v>
+        <v>0.3</v>
       </c>
       <c r="G51">
-        <v>0.5090632627797804</v>
+        <v>0.4777473486008127</v>
       </c>
       <c r="H51">
         <v>0.89375</v>
       </c>
       <c r="I51">
-        <v>0.398683924810865</v>
+        <v>0.0062169531045146</v>
       </c>
       <c r="J51">
-        <v>0.4374980827218934</v>
+        <v>0.223558685391244</v>
       </c>
       <c r="K51">
         <v>0.15</v>
@@ -3900,28 +3900,28 @@
         <v>0.0499999999995</v>
       </c>
       <c r="M51">
-        <v>0.8379997740271085</v>
+        <v>0.6486250436701073</v>
       </c>
       <c r="N51">
-        <v>0.2916986137488898</v>
+        <v>0.1978815580315132</v>
       </c>
       <c r="O51">
-        <v>0.4416666666666667</v>
+        <v>0.2666666666666667</v>
       </c>
       <c r="P51">
         <v>0.4125</v>
       </c>
       <c r="Q51">
-        <v>0.4302730232322309</v>
+        <v>0.3652723381564097</v>
       </c>
       <c r="R51">
-        <v>0.3302192279395666</v>
+        <v>0.2510063091860507</v>
       </c>
       <c r="S51">
-        <v>0.537074021757453</v>
+        <v>0.3896885709389533</v>
       </c>
       <c r="T51">
-        <v>0.999999999999999</v>
+        <v>0</v>
       </c>
     </row>
     <row r="52" spans="1:20">
@@ -3929,13 +3929,13 @@
         <v>70</v>
       </c>
       <c r="B52">
-        <v>0.1368101883432863</v>
+        <v>0.1064351308876456</v>
       </c>
       <c r="C52" t="s">
         <v>134</v>
       </c>
       <c r="D52">
-        <v>0.2666666666666667</v>
+        <v>0.1888888888888889</v>
       </c>
       <c r="E52">
         <v>0.03599311707714975</v>
@@ -3944,13 +3944,13 @@
         <v>0.15</v>
       </c>
       <c r="G52">
-        <v>0.1506975938578337</v>
+        <v>0.1240598889883222</v>
       </c>
       <c r="H52">
         <v>0.075</v>
       </c>
       <c r="I52">
-        <v>0.1877312681325749</v>
+        <v>0.07447434036172967</v>
       </c>
       <c r="J52">
         <v>0.08804392953912829</v>
@@ -3980,10 +3980,10 @@
         <v>0.1129245388483546</v>
       </c>
       <c r="S52">
-        <v>0.1229227828287388</v>
+        <v>0.08881037278696899</v>
       </c>
       <c r="T52">
-        <v>0.4827304013362672</v>
+        <v>0.08191500657628896</v>
       </c>
     </row>
     <row r="53" spans="1:20">
@@ -3991,61 +3991,61 @@
         <v>71</v>
       </c>
       <c r="B53">
-        <v>0.1855971345226895</v>
+        <v>0.1057491672647454</v>
       </c>
       <c r="C53" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="D53">
-        <v>0.3055555555555556</v>
+        <v>0.2277777777777778</v>
       </c>
       <c r="E53">
-        <v>0.05698910203882045</v>
+        <v>0</v>
       </c>
       <c r="F53">
         <v>0</v>
       </c>
       <c r="G53">
-        <v>0.1242726701289213</v>
+        <v>0.07801042140356956</v>
       </c>
       <c r="H53">
         <v>0.33375</v>
       </c>
       <c r="I53">
-        <v>0.1681849405967452</v>
+        <v>0</v>
       </c>
       <c r="J53">
-        <v>0.1944974818165595</v>
+        <v>0.1397147372678472</v>
       </c>
       <c r="K53">
         <v>0</v>
       </c>
       <c r="L53">
-        <v>0.2533002355658751</v>
+        <v>0</v>
       </c>
       <c r="M53">
         <v>0</v>
       </c>
       <c r="N53">
-        <v>0.3220952781506888</v>
+        <v>0.200568672235225</v>
       </c>
       <c r="O53">
-        <v>0.3833333333333334</v>
+        <v>0.1500000000000001</v>
       </c>
       <c r="P53">
-        <v>0.2375</v>
+        <v>0</v>
       </c>
       <c r="Q53">
-        <v>0.3142918970233541</v>
+        <v>0.07251453539124889</v>
       </c>
       <c r="R53">
-        <v>0.2334020201886976</v>
+        <v>0.0629639691001871</v>
       </c>
       <c r="S53">
-        <v>0.2469215989164576</v>
+        <v>0.1334879131259211</v>
       </c>
       <c r="T53">
-        <v>0.06018245381115107</v>
+        <v>0.03677816621792566</v>
       </c>
     </row>
     <row r="54" spans="1:20">
@@ -4115,7 +4115,7 @@
         <v>73</v>
       </c>
       <c r="B55">
-        <v>0.3958682487979567</v>
+        <v>0.2972563377480603</v>
       </c>
       <c r="C55" t="s">
         <v>135</v>
@@ -4127,10 +4127,10 @@
         <v>0.0989810719621618</v>
       </c>
       <c r="F55">
-        <v>0.25</v>
+        <v>0</v>
       </c>
       <c r="G55">
-        <v>0.2303414982206626</v>
+        <v>0.1520517127732436</v>
       </c>
       <c r="H55">
         <v>1</v>
@@ -4139,37 +4139,37 @@
         <v>0.05000000000000005</v>
       </c>
       <c r="J55">
-        <v>0.5981991663276858</v>
+        <v>0.1775105320959078</v>
       </c>
       <c r="K55">
-        <v>1</v>
+        <v>0.15</v>
       </c>
       <c r="L55">
-        <v>0.29339952886025</v>
+        <v>0.2533002355658751</v>
       </c>
       <c r="M55">
-        <v>0.5767284630504464</v>
+        <v>0.4346974152826956</v>
       </c>
       <c r="N55">
-        <v>0.400496395966067</v>
+        <v>0.2779105258733153</v>
       </c>
       <c r="O55">
-        <v>0.7166666666666667</v>
+        <v>0.2916666666666666</v>
       </c>
       <c r="P55">
         <v>0.4125</v>
       </c>
       <c r="Q55">
-        <v>0.5284805888945167</v>
+        <v>0.290395357612641</v>
       </c>
       <c r="R55">
-        <v>0.5860496136083301</v>
+        <v>0.2631477771532772</v>
       </c>
       <c r="S55">
-        <v>0.5613949993752507</v>
+        <v>0.442460962722877</v>
       </c>
       <c r="T55">
-        <v>0.7400242908201713</v>
+        <v>0.6547658145877073</v>
       </c>
     </row>
     <row r="56" spans="1:20">
@@ -4177,7 +4177,7 @@
         <v>74</v>
       </c>
       <c r="B56">
-        <v>0.2176176276547921</v>
+        <v>0.1577061434538511</v>
       </c>
       <c r="C56" t="s">
         <v>135</v>
@@ -4195,7 +4195,7 @@
         <v>0.156579570894838</v>
       </c>
       <c r="H56">
-        <v>0.68125</v>
+        <v>0.32</v>
       </c>
       <c r="I56">
         <v>0</v>
@@ -4213,7 +4213,7 @@
         <v>0.01686125637994725</v>
       </c>
       <c r="N56">
-        <v>0.1674848305087236</v>
+        <v>0.1430741414803772</v>
       </c>
       <c r="O56">
         <v>0.5</v>
@@ -4222,16 +4222,16 @@
         <v>0</v>
       </c>
       <c r="Q56">
-        <v>0.162161697116697</v>
+        <v>0.1559012686786509</v>
       </c>
       <c r="R56">
-        <v>0.1453014146213278</v>
+        <v>0.1441111794702238</v>
       </c>
       <c r="S56">
-        <v>0.2786556844147461</v>
+        <v>0.1588327160128641</v>
       </c>
       <c r="T56">
-        <v>0.2920974603874399</v>
+        <v>0.1784194920774879</v>
       </c>
     </row>
     <row r="57" spans="1:20">
@@ -4239,13 +4239,13 @@
         <v>75</v>
       </c>
       <c r="B57">
-        <v>0.2600479933211381</v>
+        <v>0.1284034201405304</v>
       </c>
       <c r="C57" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="D57">
-        <v>0.7166666666666667</v>
+        <v>0.3388888888888889</v>
       </c>
       <c r="E57">
         <v>0</v>
@@ -4254,19 +4254,19 @@
         <v>0.3</v>
       </c>
       <c r="G57">
-        <v>0.3393951659774022</v>
+        <v>0.2100120280397746</v>
       </c>
       <c r="H57">
-        <v>0.1625</v>
+        <v>0</v>
       </c>
       <c r="I57">
-        <v>0.1536305282796979</v>
+        <v>0.026970637397583</v>
       </c>
       <c r="J57">
-        <v>0.4049909389975564</v>
+        <v>0.1688727749010497</v>
       </c>
       <c r="K57">
-        <v>0.4333333333333333</v>
+        <v>0</v>
       </c>
       <c r="L57">
         <v>0</v>
@@ -4275,7 +4275,7 @@
         <v>0.8479843631296788</v>
       </c>
       <c r="N57">
-        <v>0.425289703091893</v>
+        <v>0.3185801196251216</v>
       </c>
       <c r="O57">
         <v>0.15</v>
@@ -4284,16 +4284,16 @@
         <v>0</v>
       </c>
       <c r="Q57">
-        <v>0.292393042627257</v>
+        <v>0.2650260268837983</v>
       </c>
       <c r="R57">
-        <v>0.2191674721646166</v>
+        <v>0.1049915091817301</v>
       </c>
       <c r="S57">
-        <v>0.1807008206648741</v>
+        <v>0.04679481224128626</v>
       </c>
       <c r="T57">
-        <v>0.5835867414043761</v>
+        <v>0.02507602242131295</v>
       </c>
     </row>
     <row r="58" spans="1:20">
@@ -4301,7 +4301,7 @@
         <v>76</v>
       </c>
       <c r="B58">
-        <v>0.1307205911424718</v>
+        <v>0.09995951539425274</v>
       </c>
       <c r="C58" t="s">
         <v>134</v>
@@ -4319,13 +4319,13 @@
         <v>0.02951868759574299</v>
       </c>
       <c r="H58">
-        <v>0.5962500000000001</v>
+        <v>0.42625</v>
       </c>
       <c r="I58">
         <v>0.04926936869601695</v>
       </c>
       <c r="J58">
-        <v>0.1021091197076115</v>
+        <v>0.0353454645141732</v>
       </c>
       <c r="K58">
         <v>0</v>
@@ -4337,7 +4337,7 @@
         <v>0.06698986147444755</v>
       </c>
       <c r="N58">
-        <v>0.1303899386151829</v>
+        <v>0.08784559488006487</v>
       </c>
       <c r="O58">
         <v>0</v>
@@ -4346,16 +4346,16 @@
         <v>0.15</v>
       </c>
       <c r="Q58">
-        <v>0.05494778676855472</v>
+        <v>0.04403675434796006</v>
       </c>
       <c r="R58">
-        <v>0.05439788449486715</v>
+        <v>0.03989677153147388</v>
       </c>
       <c r="S58">
-        <v>0.2319224946892007</v>
+        <v>0.1704003431927625</v>
       </c>
       <c r="T58">
-        <v>0.999999999999999</v>
+        <v>0.05349551449880097</v>
       </c>
     </row>
     <row r="59" spans="1:20">
@@ -4363,13 +4363,13 @@
         <v>77</v>
       </c>
       <c r="B59">
-        <v>0.2531681200631208</v>
+        <v>0.190282824014711</v>
       </c>
       <c r="C59" t="s">
         <v>135</v>
       </c>
       <c r="D59">
-        <v>0.6222222222222222</v>
+        <v>0.4333333333333333</v>
       </c>
       <c r="E59">
         <v>0</v>
@@ -4378,16 +4378,16 @@
         <v>0.5142857142857142</v>
       </c>
       <c r="G59">
-        <v>0.3741549118764972</v>
+        <v>0.3094633429076835</v>
       </c>
       <c r="H59">
         <v>0.14375</v>
       </c>
       <c r="I59">
-        <v>0.1856540012049723</v>
+        <v>0.008990212465861</v>
       </c>
       <c r="J59">
-        <v>0.1515301681215497</v>
+        <v>0.0515800977033492</v>
       </c>
       <c r="K59">
         <v>0.05</v>
@@ -4399,7 +4399,7 @@
         <v>0.1410507844517152</v>
       </c>
       <c r="N59">
-        <v>0.4746996098131698</v>
+        <v>0.4180982828107959</v>
       </c>
       <c r="O59">
         <v>0.05</v>
@@ -4408,16 +4408,16 @@
         <v>0</v>
       </c>
       <c r="Q59">
-        <v>0.1637921549425335</v>
+        <v>0.1492760322396745</v>
       </c>
       <c r="R59">
-        <v>0.07807513160952306</v>
+        <v>0.05671163793768748</v>
       </c>
       <c r="S59">
-        <v>0.1321813282497444</v>
+        <v>0.07110230512173854</v>
       </c>
       <c r="T59">
-        <v>0.999999999999999</v>
+        <v>0.6547658145877073</v>
       </c>
     </row>
     <row r="60" spans="1:20">
@@ -4487,7 +4487,7 @@
         <v>79</v>
       </c>
       <c r="B61">
-        <v>0.0966310426094088</v>
+        <v>0.06234333104536499</v>
       </c>
       <c r="C61" t="s">
         <v>134</v>
@@ -4496,16 +4496,16 @@
         <v>0.05</v>
       </c>
       <c r="E61">
-        <v>0.03599311707714976</v>
+        <v>0</v>
       </c>
       <c r="F61">
         <v>0</v>
       </c>
       <c r="G61">
-        <v>0.02951868759574299</v>
+        <v>0.017124238844686</v>
       </c>
       <c r="H61">
-        <v>0.42625</v>
+        <v>0.25625</v>
       </c>
       <c r="I61">
         <v>0</v>
@@ -4538,10 +4538,10 @@
         <v>0.06211262346869185</v>
       </c>
       <c r="S61">
-        <v>0.1637433976230746</v>
+        <v>0.107562423246044</v>
       </c>
       <c r="T61">
-        <v>0.7116047987426833</v>
+        <v>0.110334498653777</v>
       </c>
     </row>
     <row r="62" spans="1:20">
@@ -4549,7 +4549,7 @@
         <v>80</v>
       </c>
       <c r="B62">
-        <v>0.09278937099014428</v>
+        <v>0.06188148110040166</v>
       </c>
       <c r="C62" t="s">
         <v>134</v>
@@ -4567,13 +4567,13 @@
         <v>0</v>
       </c>
       <c r="H62">
-        <v>0.42625</v>
+        <v>0.25625</v>
       </c>
       <c r="I62">
         <v>0.026970637397583</v>
       </c>
       <c r="J62">
-        <v>0.2437626435372299</v>
+        <v>0.1769989883437917</v>
       </c>
       <c r="K62">
         <v>0.15</v>
@@ -4585,7 +4585,7 @@
         <v>0</v>
       </c>
       <c r="N62">
-        <v>0.133606503111805</v>
+        <v>0.07471246994259101</v>
       </c>
       <c r="O62">
         <v>0</v>
@@ -4594,16 +4594,16 @@
         <v>0.15</v>
       </c>
       <c r="Q62">
-        <v>0.03426506931523929</v>
+        <v>0.01916095325953799</v>
       </c>
       <c r="R62">
-        <v>0.09934003211573268</v>
+        <v>0.08404172841956252</v>
       </c>
       <c r="S62">
-        <v>0.1855787419802886</v>
+        <v>0.1237629622008033</v>
       </c>
       <c r="T62">
-        <v>0.1784194920774879</v>
+        <v>0.1499999999999999</v>
       </c>
     </row>
     <row r="63" spans="1:20">
@@ -4611,13 +4611,13 @@
         <v>81</v>
       </c>
       <c r="B63">
-        <v>0.20098397421881</v>
+        <v>0.1545929461401455</v>
       </c>
       <c r="C63" t="s">
         <v>135</v>
       </c>
       <c r="D63">
-        <v>0.1888888888888889</v>
+        <v>0</v>
       </c>
       <c r="E63">
         <v>0</v>
@@ -4626,10 +4626,10 @@
         <v>0.5</v>
       </c>
       <c r="G63">
-        <v>0.2212711398636518</v>
+        <v>0.156579570894838</v>
       </c>
       <c r="H63">
-        <v>0.51125</v>
+        <v>0.42625</v>
       </c>
       <c r="I63">
         <v>0</v>
@@ -4662,7 +4662,7 @@
         <v>0.03187584288771285</v>
       </c>
       <c r="S63">
-        <v>0.1806968085739683</v>
+        <v>0.152606321385453</v>
       </c>
       <c r="T63">
         <v>0</v>
@@ -4673,10 +4673,10 @@
         <v>82</v>
       </c>
       <c r="B64">
-        <v>0.1526869294664921</v>
+        <v>0.1051809584859148</v>
       </c>
       <c r="C64" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="D64">
         <v>0.15</v>
@@ -4691,7 +4691,7 @@
         <v>0.1107410365535664</v>
       </c>
       <c r="H64">
-        <v>0.3625</v>
+        <v>0.075</v>
       </c>
       <c r="I64">
         <v>0.1105561215150873</v>
@@ -4724,7 +4724,7 @@
         <v>0.1127694025667084</v>
       </c>
       <c r="S64">
-        <v>0.1946328223794179</v>
+        <v>0.09962088041826316</v>
       </c>
       <c r="T64">
         <v>0.1499999999999999</v>
@@ -4735,7 +4735,7 @@
         <v>83</v>
       </c>
       <c r="B65">
-        <v>0.08459174424083132</v>
+        <v>0.08320114993102326</v>
       </c>
       <c r="C65" t="s">
         <v>134</v>
@@ -4768,10 +4768,10 @@
         <v>0.0687416456475</v>
       </c>
       <c r="M65">
-        <v>0.2395196679081972</v>
+        <v>0.09987139490549971</v>
       </c>
       <c r="N65">
-        <v>0.1572364194323185</v>
+        <v>0.120092269149797</v>
       </c>
       <c r="O65">
         <v>0</v>
@@ -4780,13 +4780,13 @@
         <v>0</v>
       </c>
       <c r="Q65">
-        <v>0.126774882865943</v>
+        <v>0.08705882974584583</v>
       </c>
       <c r="R65">
-        <v>0.07029842171486356</v>
+        <v>0.06274758985815281</v>
       </c>
       <c r="S65">
-        <v>0.08133350454617876</v>
+        <v>0.07855231592656262</v>
       </c>
       <c r="T65">
         <v>0</v>
@@ -4859,34 +4859,34 @@
         <v>85</v>
       </c>
       <c r="B67">
-        <v>0.5509620433626017</v>
+        <v>0.3589518956831894</v>
       </c>
       <c r="C67" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="D67">
-        <v>0.2666666666666667</v>
+        <v>0</v>
       </c>
       <c r="E67">
-        <v>0.620353584076456</v>
+        <v>0.380399470228791</v>
       </c>
       <c r="F67">
         <v>0.2714285714285715</v>
       </c>
       <c r="G67">
-        <v>0.3899521415673728</v>
+        <v>0.2159932093886675</v>
       </c>
       <c r="H67">
-        <v>1</v>
+        <v>0.8300000000000001</v>
       </c>
       <c r="I67">
-        <v>0.3691428536760846</v>
+        <v>0.08206378097959272</v>
       </c>
       <c r="J67">
-        <v>0.7388967254832586</v>
+        <v>0.3556028192495407</v>
       </c>
       <c r="K67">
-        <v>0.7166666666666667</v>
+        <v>0</v>
       </c>
       <c r="L67">
         <v>0.5685538785463751</v>
@@ -4895,7 +4895,7 @@
         <v>0.8134101921482488</v>
       </c>
       <c r="N67">
-        <v>0.65618326280362</v>
+        <v>0.5712121680202531</v>
       </c>
       <c r="O67">
         <v>0.8583333333333334</v>
@@ -4904,16 +4904,16 @@
         <v>0.7875</v>
       </c>
       <c r="Q67">
-        <v>0.7275287732962832</v>
+        <v>0.7057368665796813</v>
       </c>
       <c r="R67">
-        <v>0.7338869461675841</v>
+        <v>0.5508612394612068</v>
       </c>
       <c r="S67">
-        <v>0.7119719451578305</v>
+        <v>0.5019105819777113</v>
       </c>
       <c r="T67">
-        <v>0.999999999999999</v>
+        <v>0.05349551449880097</v>
       </c>
     </row>
     <row r="68" spans="1:20">
@@ -4921,7 +4921,7 @@
         <v>86</v>
       </c>
       <c r="B68">
-        <v>0.1036278438539662</v>
+        <v>0.09489765874627426</v>
       </c>
       <c r="C68" t="s">
         <v>134</v>
@@ -4942,10 +4942,10 @@
         <v>0.075</v>
       </c>
       <c r="I68">
-        <v>0.1704356749308377</v>
+        <v>0.1279323617523907</v>
       </c>
       <c r="J68">
-        <v>0.1420446242832497</v>
+        <v>0.07920824292471959</v>
       </c>
       <c r="K68">
         <v>0</v>
@@ -4957,7 +4957,7 @@
         <v>0.1214010459356202</v>
       </c>
       <c r="N68">
-        <v>0.1540260943756797</v>
+        <v>0.1344975431530026</v>
       </c>
       <c r="O68">
         <v>0</v>
@@ -4966,16 +4966,16 @@
         <v>0</v>
       </c>
       <c r="Q68">
-        <v>0.0868232831015696</v>
+        <v>0.08181494035113271</v>
       </c>
       <c r="R68">
-        <v>0.05537055797318824</v>
+        <v>0.04272264926067026</v>
       </c>
       <c r="S68">
-        <v>0.09651465115436603</v>
+        <v>0.07905428093898212</v>
       </c>
       <c r="T68">
-        <v>0.6263463225102193</v>
+        <v>0.02507602242131295</v>
       </c>
     </row>
     <row r="69" spans="1:20">
@@ -4983,7 +4983,7 @@
         <v>87</v>
       </c>
       <c r="B69">
-        <v>0.8332644607870843</v>
+        <v>0.8248139725239658</v>
       </c>
       <c r="C69" t="s">
         <v>137</v>
@@ -5010,7 +5010,7 @@
         <v>0.7761453914102374</v>
       </c>
       <c r="K69">
-        <v>1</v>
+        <v>0.7166666666666667</v>
       </c>
       <c r="L69">
         <v>0.8052320039887501</v>
@@ -5019,7 +5019,7 @@
         <v>1</v>
       </c>
       <c r="N69">
-        <v>0.7447709152897485</v>
+        <v>0.6756618618521892</v>
       </c>
       <c r="O69">
         <v>0.8583333333333334</v>
@@ -5028,13 +5028,13 @@
         <v>1</v>
       </c>
       <c r="Q69">
-        <v>0.6805968520853529</v>
+        <v>0.6628729655140015</v>
       </c>
       <c r="R69">
-        <v>0.8459425546807251</v>
+        <v>0.8000569822086777</v>
       </c>
       <c r="S69">
-        <v>0.821923152396313</v>
+        <v>0.8050221758700761</v>
       </c>
       <c r="T69">
         <v>0.999999999999999</v>
@@ -5045,34 +5045,34 @@
         <v>88</v>
       </c>
       <c r="B70">
-        <v>0.1561077345577246</v>
+        <v>0.08369781759172538</v>
       </c>
       <c r="C70" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="D70">
-        <v>0.3833333333333334</v>
+        <v>0.2277777777777778</v>
       </c>
       <c r="E70">
-        <v>0.05698910203882045</v>
+        <v>0</v>
       </c>
       <c r="F70">
         <v>0</v>
       </c>
       <c r="G70">
-        <v>0.1509103749984329</v>
+        <v>0.07801042140356956</v>
       </c>
       <c r="H70">
         <v>0.075</v>
       </c>
       <c r="I70">
-        <v>0.2042629901966475</v>
+        <v>0.0300023387141979</v>
       </c>
       <c r="J70">
-        <v>0.1665978183725157</v>
+        <v>0.01325488894988225</v>
       </c>
       <c r="K70">
-        <v>0.1500000000000001</v>
+        <v>0</v>
       </c>
       <c r="L70">
         <v>0.081258354351</v>
@@ -5081,7 +5081,7 @@
         <v>0.632292446191752</v>
       </c>
       <c r="N70">
-        <v>0.1420203210768662</v>
+        <v>0.1069276371069552</v>
       </c>
       <c r="O70">
         <v>0.3250000000000001</v>
@@ -5090,16 +5090,16 @@
         <v>0.15</v>
       </c>
       <c r="Q70">
-        <v>0.3288334600856089</v>
+        <v>0.3198334995995497</v>
       </c>
       <c r="R70">
-        <v>0.2036126505994817</v>
+        <v>0.1508514741528101</v>
       </c>
       <c r="S70">
-        <v>0.1613050941170163</v>
+        <v>0.08938521377988121</v>
       </c>
       <c r="T70">
-        <v>0.4166626484921777</v>
+        <v>0</v>
       </c>
     </row>
     <row r="71" spans="1:20">
@@ -5223,7 +5223,7 @@
         <v>0.06689232732203816</v>
       </c>
       <c r="T72">
-        <v>0.167173482808753</v>
+        <v>0.05349551449880097</v>
       </c>
     </row>
     <row r="73" spans="1:20">
@@ -5231,34 +5231,34 @@
         <v>91</v>
       </c>
       <c r="B73">
-        <v>0.510089418170998</v>
+        <v>0.1173045400650294</v>
       </c>
       <c r="C73" t="s">
-        <v>136</v>
+        <v>134</v>
       </c>
       <c r="D73">
-        <v>0.9055555555555556</v>
+        <v>0</v>
       </c>
       <c r="E73">
-        <v>0.239954113847665</v>
+        <v>0</v>
       </c>
       <c r="F73">
         <v>0.35</v>
       </c>
       <c r="G73">
-        <v>0.5023743503760797</v>
+        <v>0.1096056996263866</v>
       </c>
       <c r="H73">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I73">
         <v>0</v>
       </c>
       <c r="J73">
-        <v>0.4593819680971288</v>
+        <v>0.02492968019641535</v>
       </c>
       <c r="K73">
-        <v>0.4333333333333333</v>
+        <v>0</v>
       </c>
       <c r="L73">
         <v>0.54172236234</v>
@@ -5267,7 +5267,7 @@
         <v>0.8354884983201507</v>
       </c>
       <c r="N73">
-        <v>0.6533060561235416</v>
+        <v>0.1750158741597591</v>
       </c>
       <c r="O73">
         <v>1</v>
@@ -5276,16 +5276,16 @@
         <v>0.15</v>
       </c>
       <c r="Q73">
-        <v>0.503887215276854</v>
+        <v>0.381223678277663</v>
       </c>
       <c r="R73">
-        <v>0.5085895556591504</v>
+        <v>0.3393798971584805</v>
       </c>
       <c r="S73">
-        <v>0.5178044859659162</v>
+        <v>0.1250033805036722</v>
       </c>
       <c r="T73">
-        <v>0.999999999999999</v>
+        <v>0.886322031690047</v>
       </c>
     </row>
     <row r="74" spans="1:20">
@@ -5293,7 +5293,7 @@
         <v>92</v>
       </c>
       <c r="B74">
-        <v>0.09675143097494646</v>
+        <v>0.08521458655243916</v>
       </c>
       <c r="C74" t="s">
         <v>134</v>
@@ -5314,10 +5314,10 @@
         <v>0.15</v>
       </c>
       <c r="I74">
-        <v>0.05989291775225067</v>
+        <v>0.026970637397583</v>
       </c>
       <c r="J74">
-        <v>0.1426633145049839</v>
+        <v>0.04722811406583174</v>
       </c>
       <c r="K74">
         <v>0.15</v>
@@ -5326,10 +5326,10 @@
         <v>0</v>
       </c>
       <c r="M74">
-        <v>0.6251905627096774</v>
+        <v>0.4157181532056312</v>
       </c>
       <c r="N74">
-        <v>0.2305472451170721</v>
+        <v>0.03879327921645105</v>
       </c>
       <c r="O74">
         <v>0.15</v>
@@ -5338,13 +5338,13 @@
         <v>0.15</v>
       </c>
       <c r="Q74">
-        <v>0.1942840407607035</v>
+        <v>0.09982137034312417</v>
       </c>
       <c r="R74">
-        <v>0.134117715088796</v>
+        <v>0.09839510355161622</v>
       </c>
       <c r="S74">
-        <v>0.1170103030856985</v>
+        <v>0.09393661424068393</v>
       </c>
       <c r="T74">
         <v>0.008358674140437649</v>
@@ -5417,7 +5417,7 @@
         <v>94</v>
       </c>
       <c r="B76">
-        <v>0.2136315871709526</v>
+        <v>0.2020650627708691</v>
       </c>
       <c r="C76" t="s">
         <v>135</v>
@@ -5438,7 +5438,7 @@
         <v>0</v>
       </c>
       <c r="I76">
-        <v>0.1693634000949546</v>
+        <v>0.09255915102923779</v>
       </c>
       <c r="J76">
         <v>0</v>
@@ -5468,7 +5468,7 @@
         <v>0.01335670265682246</v>
       </c>
       <c r="S76">
-        <v>0.05593105173929545</v>
+        <v>0.03279800293912848</v>
       </c>
       <c r="T76">
         <v>0</v>
@@ -5479,7 +5479,7 @@
         <v>95</v>
       </c>
       <c r="B77">
-        <v>0.2712443340740192</v>
+        <v>0.204065733128296</v>
       </c>
       <c r="C77" t="s">
         <v>135</v>
@@ -5488,13 +5488,13 @@
         <v>0.4333333333333333</v>
       </c>
       <c r="E77">
-        <v>0.379646415923544</v>
+        <v>0</v>
       </c>
       <c r="F77">
         <v>0</v>
       </c>
       <c r="G77">
-        <v>0.2791436220606034</v>
+        <v>0.1484100699872787</v>
       </c>
       <c r="H77">
         <v>0.6174999999999999</v>
@@ -5515,7 +5515,7 @@
         <v>0.1744698545147154</v>
       </c>
       <c r="N77">
-        <v>0.2199825144731298</v>
+        <v>0.1962692737027361</v>
       </c>
       <c r="O77">
         <v>0.15</v>
@@ -5524,16 +5524,16 @@
         <v>0</v>
       </c>
       <c r="Q77">
-        <v>0.1744691110609493</v>
+        <v>0.1227225061560964</v>
       </c>
       <c r="R77">
-        <v>0.1054079997625611</v>
+        <v>0.09556991460312543</v>
       </c>
       <c r="S77">
-        <v>0.2633450460874349</v>
+        <v>0.2597213962693133</v>
       </c>
       <c r="T77">
-        <v>0.1968085751864507</v>
+        <v>0.1617021437966126</v>
       </c>
     </row>
     <row r="78" spans="1:20">
@@ -5541,7 +5541,7 @@
         <v>96</v>
       </c>
       <c r="B78">
-        <v>0.5110570238180594</v>
+        <v>0.465343845173425</v>
       </c>
       <c r="C78" t="s">
         <v>136</v>
@@ -5559,16 +5559,16 @@
         <v>0.3428640638679554</v>
       </c>
       <c r="H78">
-        <v>1</v>
+        <v>0.915</v>
       </c>
       <c r="I78">
         <v>0.08190358204299537</v>
       </c>
       <c r="J78">
-        <v>0.7899476849709188</v>
+        <v>0.4635058230376705</v>
       </c>
       <c r="K78">
-        <v>0.7166666666666667</v>
+        <v>0</v>
       </c>
       <c r="L78">
         <v>0.99999999999</v>
@@ -5577,7 +5577,7 @@
         <v>0.8603517269973024</v>
       </c>
       <c r="N78">
-        <v>0.7947493550139614</v>
+        <v>0.719809912857948</v>
       </c>
       <c r="O78">
         <v>1</v>
@@ -5586,13 +5586,13 @@
         <v>1</v>
       </c>
       <c r="Q78">
-        <v>0.7977392621198238</v>
+        <v>0.7785200989794461</v>
       </c>
       <c r="R78">
-        <v>0.879933220750494</v>
+        <v>0.7079785024490545</v>
       </c>
       <c r="S78">
-        <v>0.6792499837681634</v>
+        <v>0.5878236264788945</v>
       </c>
       <c r="T78">
         <v>0.7685905033694724</v>
@@ -5603,13 +5603,13 @@
         <v>97</v>
       </c>
       <c r="B79">
-        <v>0.3850076273922133</v>
+        <v>0.3484885889691788</v>
       </c>
       <c r="C79" t="s">
         <v>135</v>
       </c>
       <c r="D79">
-        <v>0.4222222222222222</v>
+        <v>0.3444444444444444</v>
       </c>
       <c r="E79">
         <v>0</v>
@@ -5618,16 +5618,16 @@
         <v>0.5</v>
       </c>
       <c r="G79">
-        <v>0.3011842544721864</v>
+        <v>0.2745465496026749</v>
       </c>
       <c r="H79">
-        <v>1</v>
+        <v>0.915</v>
       </c>
       <c r="I79">
         <v>0.026970637397583</v>
       </c>
       <c r="J79">
-        <v>0.5773565727166654</v>
+        <v>0.3634171753860159</v>
       </c>
       <c r="K79">
         <v>0</v>
@@ -5639,7 +5639,7 @@
         <v>0.2563645918314487</v>
       </c>
       <c r="N79">
-        <v>0.6700428669736299</v>
+        <v>0.4672030165962475</v>
       </c>
       <c r="O79">
         <v>0.15</v>
@@ -5648,16 +5648,16 @@
         <v>0.325</v>
       </c>
       <c r="Q79">
-        <v>0.4092749328142589</v>
+        <v>0.3572541002110915</v>
       </c>
       <c r="R79">
-        <v>0.3535734157703002</v>
+        <v>0.3038627056174113</v>
       </c>
       <c r="S79">
-        <v>0.4688310003122402</v>
+        <v>0.4224306283356828</v>
       </c>
       <c r="T79">
-        <v>0.999999999999999</v>
+        <v>0.832826517191246</v>
       </c>
     </row>
     <row r="80" spans="1:20">
@@ -5665,13 +5665,13 @@
         <v>98</v>
       </c>
       <c r="B80">
-        <v>0.1178504504813622</v>
+        <v>0.1111910242639843</v>
       </c>
       <c r="C80" t="s">
         <v>134</v>
       </c>
       <c r="D80">
-        <v>0.2277777777777778</v>
+        <v>0.1888888888888889</v>
       </c>
       <c r="E80">
         <v>0</v>
@@ -5680,7 +5680,7 @@
         <v>0.15</v>
       </c>
       <c r="G80">
-        <v>0.124984292672021</v>
+        <v>0.1116654402372652</v>
       </c>
       <c r="H80">
         <v>0.15</v>
@@ -5727,7 +5727,7 @@
         <v>99</v>
       </c>
       <c r="B81">
-        <v>0.02621539190980106</v>
+        <v>0.003131375757495653</v>
       </c>
       <c r="C81" t="s">
         <v>134</v>
@@ -5748,7 +5748,7 @@
         <v>0</v>
       </c>
       <c r="I81">
-        <v>0.1740759298083705</v>
+        <v>0.02079301917136905</v>
       </c>
       <c r="J81">
         <v>0</v>
@@ -5778,7 +5778,7 @@
         <v>0</v>
       </c>
       <c r="S81">
-        <v>0.05243078381960212</v>
+        <v>0.006262751514991307</v>
       </c>
       <c r="T81">
         <v>0.02507602242131295</v>
@@ -5789,61 +5789,61 @@
         <v>100</v>
       </c>
       <c r="B82">
-        <v>0.6657515254662403</v>
+        <v>0.04980188877090345</v>
       </c>
       <c r="C82" t="s">
-        <v>136</v>
+        <v>134</v>
       </c>
       <c r="D82">
-        <v>0.9055555555555556</v>
+        <v>0</v>
       </c>
       <c r="E82">
-        <v>0.239954113847665</v>
+        <v>0</v>
       </c>
       <c r="F82">
-        <v>0.8785714285714286</v>
+        <v>0</v>
       </c>
       <c r="G82">
-        <v>0.6679013253220513</v>
+        <v>0</v>
       </c>
       <c r="H82">
-        <v>0.575</v>
+        <v>0.075</v>
       </c>
       <c r="I82">
-        <v>0.4765638294127857</v>
+        <v>0.026970637397583</v>
       </c>
       <c r="J82">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K82">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L82">
-        <v>0.99999999999</v>
+        <v>0</v>
       </c>
       <c r="M82">
-        <v>1</v>
+        <v>0.8106252696429989</v>
       </c>
       <c r="N82">
-        <v>1</v>
+        <v>0.3443739629109572</v>
       </c>
       <c r="O82">
-        <v>0.5</v>
+        <v>0</v>
       </c>
       <c r="P82">
-        <v>1</v>
+        <v>0.7875</v>
       </c>
       <c r="Q82">
-        <v>0.859492166613073</v>
+        <v>0.2635646785555469</v>
       </c>
       <c r="R82">
-        <v>0.8960452407632044</v>
+        <v>0.181073649646545</v>
       </c>
       <c r="S82">
-        <v>0.6636017256104293</v>
+        <v>0.0996037775418069</v>
       </c>
       <c r="T82">
-        <v>0.9147415237675349</v>
+        <v>0.6012703000889064</v>
       </c>
     </row>
     <row r="83" spans="1:20">
@@ -5913,22 +5913,22 @@
         <v>102</v>
       </c>
       <c r="B84">
-        <v>0.1968235753790364</v>
+        <v>0.1534455173107375</v>
       </c>
       <c r="C84" t="s">
         <v>135</v>
       </c>
       <c r="D84">
-        <v>0.5277777777777778</v>
+        <v>0.3388888888888889</v>
       </c>
       <c r="E84">
-        <v>0.05698910203882045</v>
+        <v>0</v>
       </c>
       <c r="F84">
         <v>0.05</v>
       </c>
       <c r="G84">
-        <v>0.2160383554170096</v>
+        <v>0.1317222425923556</v>
       </c>
       <c r="H84">
         <v>0.43125</v>
@@ -5949,7 +5949,7 @@
         <v>0.332904649684999</v>
       </c>
       <c r="N84">
-        <v>0.3178901607516829</v>
+        <v>0.182026898689623</v>
       </c>
       <c r="O84">
         <v>0</v>
@@ -5958,13 +5958,13 @@
         <v>0</v>
       </c>
       <c r="Q84">
-        <v>0.1534961780266285</v>
+        <v>0.1186523344746774</v>
       </c>
       <c r="R84">
-        <v>0.09527054397969228</v>
+        <v>0.08864601854896201</v>
       </c>
       <c r="S84">
-        <v>0.1776087953410632</v>
+        <v>0.1751687920291194</v>
       </c>
       <c r="T84">
         <v>0.05349551449880097</v>
@@ -5975,7 +5975,7 @@
         <v>103</v>
       </c>
       <c r="B85">
-        <v>0.05478894962582694</v>
+        <v>0.0546824815763732</v>
       </c>
       <c r="C85" t="s">
         <v>134</v>
@@ -6011,7 +6011,7 @@
         <v>0.1633070482397685</v>
       </c>
       <c r="N85">
-        <v>0.2387258652307927</v>
+        <v>0.2268692448455959</v>
       </c>
       <c r="O85">
         <v>0.05</v>
@@ -6020,16 +6020,16 @@
         <v>0</v>
       </c>
       <c r="Q85">
-        <v>0.1080852054831898</v>
+        <v>0.1050444259561388</v>
       </c>
       <c r="R85">
-        <v>0.06204812178602083</v>
+        <v>0.06147000756977028</v>
       </c>
       <c r="S85">
-        <v>0.04694607089371865</v>
+        <v>0.04673313479481117</v>
       </c>
       <c r="T85">
-        <v>0.110334498653777</v>
+        <v>0.08191500657628896</v>
       </c>
     </row>
     <row r="86" spans="1:20">
@@ -6037,34 +6037,34 @@
         <v>104</v>
       </c>
       <c r="B86">
-        <v>0.6479703100793165</v>
+        <v>0.4041993795168871</v>
       </c>
       <c r="C86" t="s">
         <v>136</v>
       </c>
       <c r="D86">
-        <v>1</v>
+        <v>0.8111111111111111</v>
       </c>
       <c r="E86">
-        <v>0.5686102805785802</v>
+        <v>0.379646415923544</v>
       </c>
       <c r="F86">
         <v>1</v>
       </c>
       <c r="G86">
-        <v>0.85144832669977</v>
+        <v>0.721685901787907</v>
       </c>
       <c r="H86">
-        <v>0.68125</v>
+        <v>0</v>
       </c>
       <c r="I86">
-        <v>0.2945357985243265</v>
+        <v>0.0083756909803812</v>
       </c>
       <c r="J86">
-        <v>0.366036652087143</v>
+        <v>0.0766958423681972</v>
       </c>
       <c r="K86">
-        <v>0.4333333333333333</v>
+        <v>0</v>
       </c>
       <c r="L86">
         <v>0.650563301281875</v>
@@ -6073,7 +6073,7 @@
         <v>0.7632815870537486</v>
       </c>
       <c r="N86">
-        <v>0.4809830652507309</v>
+        <v>0.3325456097930625</v>
       </c>
       <c r="O86">
         <v>0.15</v>
@@ -6082,16 +6082,16 @@
         <v>0.15</v>
       </c>
       <c r="Q86">
-        <v>0.3889222148736857</v>
+        <v>0.350853561164678</v>
       </c>
       <c r="R86">
-        <v>0.3546902326100045</v>
+        <v>0.2285733516848029</v>
       </c>
       <c r="S86">
-        <v>0.4444922934588629</v>
+        <v>0.08671285724586721</v>
       </c>
       <c r="T86">
-        <v>0.609628974229344</v>
+        <v>0.008358674140437649</v>
       </c>
     </row>
     <row r="87" spans="1:20">
@@ -6099,7 +6099,7 @@
         <v>105</v>
       </c>
       <c r="B87">
-        <v>0.107506819575274</v>
+        <v>0.09193388632897766</v>
       </c>
       <c r="C87" t="s">
         <v>134</v>
@@ -6117,10 +6117,10 @@
         <v>0.07801042140356956</v>
       </c>
       <c r="H87">
-        <v>0.255</v>
+        <v>0.22</v>
       </c>
       <c r="I87">
-        <v>0.1204317770738412</v>
+        <v>0.05542670985974579</v>
       </c>
       <c r="J87">
         <v>0.07478904058924604</v>
@@ -6150,10 +6150,10 @@
         <v>0.04468376988887508</v>
       </c>
       <c r="S87">
-        <v>0.1370032177469784</v>
+        <v>0.1058573512543858</v>
       </c>
       <c r="T87">
-        <v>0.2068389841549759</v>
+        <v>0.05349551449880097</v>
       </c>
     </row>
     <row r="88" spans="1:20">
@@ -6161,31 +6161,31 @@
         <v>106</v>
       </c>
       <c r="B88">
-        <v>0.4981346458379184</v>
+        <v>0.3592281362834345</v>
       </c>
       <c r="C88" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="D88">
         <v>0.6222222222222222</v>
       </c>
       <c r="E88">
-        <v>0.4793805421909528</v>
+        <v>0.380399470228791</v>
       </c>
       <c r="F88">
         <v>0.8785714285714286</v>
       </c>
       <c r="G88">
-        <v>0.6533119184967556</v>
+        <v>0.6192271844313489</v>
       </c>
       <c r="H88">
-        <v>0.6799999999999999</v>
+        <v>0</v>
       </c>
       <c r="I88">
         <v>0.0353463283779642</v>
       </c>
       <c r="J88">
-        <v>0.4477941999360922</v>
+        <v>0.1906583907875988</v>
       </c>
       <c r="K88">
         <v>0.4333333333333333</v>
@@ -6197,7 +6197,7 @@
         <v>0.9301758634986512</v>
       </c>
       <c r="N88">
-        <v>0.3221311582537183</v>
+        <v>0.2455165326690076</v>
       </c>
       <c r="O88">
         <v>0.05</v>
@@ -6206,13 +6206,13 @@
         <v>0.05</v>
       </c>
       <c r="Q88">
-        <v>0.3409267074813404</v>
+        <v>0.3212779224665542</v>
       </c>
       <c r="R88">
-        <v>0.2920959477408867</v>
+        <v>0.2404996864129976</v>
       </c>
       <c r="S88">
-        <v>0.3429573731790811</v>
+        <v>0.09922908813552016</v>
       </c>
       <c r="T88">
         <v>0.1499999999999999</v>
@@ -6223,7 +6223,7 @@
         <v>107</v>
       </c>
       <c r="B89">
-        <v>0.006780420299290962</v>
+        <v>0.006529907241752744</v>
       </c>
       <c r="C89" t="s">
         <v>134</v>
@@ -6259,7 +6259,7 @@
         <v>0</v>
       </c>
       <c r="N89">
-        <v>0.05518391871991388</v>
+        <v>0.0272859884018037</v>
       </c>
       <c r="O89">
         <v>0</v>
@@ -6268,13 +6268,13 @@
         <v>0</v>
       </c>
       <c r="Q89">
-        <v>0.0141526105091011</v>
+        <v>0.006997835151334108</v>
       </c>
       <c r="R89">
-        <v>0.01438642054524275</v>
+        <v>0.0130261518011238</v>
       </c>
       <c r="S89">
-        <v>0.01356084059858192</v>
+        <v>0.01305981448350549</v>
       </c>
       <c r="T89">
         <v>0</v>
@@ -6409,7 +6409,7 @@
         <v>110</v>
       </c>
       <c r="B92">
-        <v>0.2644509841267706</v>
+        <v>0.248590329229676</v>
       </c>
       <c r="C92" t="s">
         <v>135</v>
@@ -6427,13 +6427,13 @@
         <v>0.1640680270767625</v>
       </c>
       <c r="H92">
-        <v>0.7875</v>
+        <v>0.7025</v>
       </c>
       <c r="I92">
         <v>0.05845841117636069</v>
       </c>
       <c r="J92">
-        <v>0.1813509719813091</v>
+        <v>0.1538600551369522</v>
       </c>
       <c r="K92">
         <v>0.05</v>
@@ -6445,7 +6445,7 @@
         <v>0.5151246271011529</v>
       </c>
       <c r="N92">
-        <v>0.184260717249364</v>
+        <v>0.08703346242142125</v>
       </c>
       <c r="O92">
         <v>0.3250000000000001</v>
@@ -6454,16 +6454,16 @@
         <v>0.325</v>
       </c>
       <c r="Q92">
-        <v>0.3560308010096223</v>
+        <v>0.3310956477916535</v>
       </c>
       <c r="R92">
-        <v>0.2361381196535184</v>
+        <v>0.22628056062152</v>
       </c>
       <c r="S92">
-        <v>0.3648339411767788</v>
+        <v>0.3331126313825895</v>
       </c>
       <c r="T92">
-        <v>0.2636779683099519</v>
+        <v>0.2352584762324639</v>
       </c>
     </row>
     <row r="93" spans="1:20">
@@ -6471,7 +6471,7 @@
         <v>111</v>
       </c>
       <c r="B93">
-        <v>0.2902679162046626</v>
+        <v>0.2842608868316684</v>
       </c>
       <c r="C93" t="s">
         <v>135</v>
@@ -6504,10 +6504,10 @@
         <v>0.499999999995</v>
       </c>
       <c r="M93">
-        <v>0.667095350315001</v>
+        <v>0.332904649684999</v>
       </c>
       <c r="N93">
-        <v>0.6968693278563781</v>
+        <v>0.3096143093510396</v>
       </c>
       <c r="O93">
         <v>0.5</v>
@@ -6516,16 +6516,16 @@
         <v>0.5</v>
       </c>
       <c r="Q93">
-        <v>0.4385003672992582</v>
+        <v>0.2669366725616098</v>
       </c>
       <c r="R93">
-        <v>0.4883076653060435</v>
+        <v>0.4556899072482946</v>
       </c>
       <c r="S93">
-        <v>0.5805358324093253</v>
+        <v>0.5685217736633368</v>
       </c>
       <c r="T93">
-        <v>0.999999999999999</v>
+        <v>0</v>
       </c>
     </row>
     <row r="94" spans="1:20">
@@ -6533,13 +6533,13 @@
         <v>112</v>
       </c>
       <c r="B94">
-        <v>0.2280631209161295</v>
+        <v>0.1435847446794113</v>
       </c>
       <c r="C94" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="D94">
-        <v>0.3444444444444444</v>
+        <v>0</v>
       </c>
       <c r="E94">
         <v>0.0989810719621618</v>
@@ -6548,19 +6548,19 @@
         <v>0.15</v>
       </c>
       <c r="G94">
-        <v>0.199025584041695</v>
+        <v>0.08105860533385811</v>
       </c>
       <c r="H94">
         <v>0.28125</v>
       </c>
       <c r="I94">
-        <v>0.2575590618110924</v>
+        <v>0.2148555525982526</v>
       </c>
       <c r="J94">
-        <v>0.2881914499835848</v>
+        <v>0.1252257483456379</v>
       </c>
       <c r="K94">
-        <v>0.1500000000000001</v>
+        <v>0</v>
       </c>
       <c r="L94">
         <v>0.081258354351</v>
@@ -6569,25 +6569,25 @@
         <v>0.296326064495677</v>
       </c>
       <c r="N94">
-        <v>0.3412615530421345</v>
+        <v>0.2260670351258871</v>
       </c>
       <c r="O94">
-        <v>0.2916666666666666</v>
+        <v>0</v>
       </c>
       <c r="P94">
         <v>0.4125</v>
       </c>
       <c r="Q94">
-        <v>0.1726584714401324</v>
+        <v>0.1431153874644016</v>
       </c>
       <c r="R94">
-        <v>0.2350582453273247</v>
+        <v>0.1315428613120453</v>
       </c>
       <c r="S94">
-        <v>0.257100657790564</v>
+        <v>0.2061108840249646</v>
       </c>
       <c r="T94">
-        <v>0.832826517191246</v>
+        <v>0</v>
       </c>
     </row>
     <row r="95" spans="1:20">
@@ -6595,7 +6595,7 @@
         <v>113</v>
       </c>
       <c r="B95">
-        <v>0.0685395424140734</v>
+        <v>0.05449429881981573</v>
       </c>
       <c r="C95" t="s">
         <v>134</v>
@@ -6613,7 +6613,7 @@
         <v>0</v>
       </c>
       <c r="H95">
-        <v>0.33</v>
+        <v>0.245</v>
       </c>
       <c r="I95">
         <v>0.04776365656895205</v>
@@ -6646,10 +6646,10 @@
         <v>0.03702053748893253</v>
       </c>
       <c r="S95">
-        <v>0.1370790848281468</v>
+        <v>0.1089885976396315</v>
       </c>
       <c r="T95">
-        <v>0.1734042875932253</v>
+        <v>0.1249239775786869</v>
       </c>
     </row>
     <row r="96" spans="1:20">
@@ -6657,7 +6657,7 @@
         <v>114</v>
       </c>
       <c r="B96">
-        <v>0.1277209220253125</v>
+        <v>0.1136756784310549</v>
       </c>
       <c r="C96" t="s">
         <v>134</v>
@@ -6675,7 +6675,7 @@
         <v>0.051372716534058</v>
       </c>
       <c r="H96">
-        <v>0.6174999999999999</v>
+        <v>0.5325</v>
       </c>
       <c r="I96">
         <v>0</v>
@@ -6708,10 +6708,10 @@
         <v>0</v>
       </c>
       <c r="S96">
-        <v>0.2040691275165671</v>
+        <v>0.1759786403280518</v>
       </c>
       <c r="T96">
-        <v>0.05349551449880097</v>
+        <v>0.02507602242131295</v>
       </c>
     </row>
     <row r="97" spans="1:20">
@@ -6719,7 +6719,7 @@
         <v>115</v>
       </c>
       <c r="B97">
-        <v>0.1401022923537543</v>
+        <v>0.1023211796921592</v>
       </c>
       <c r="C97" t="s">
         <v>134</v>
@@ -6740,10 +6740,10 @@
         <v>0.3125</v>
       </c>
       <c r="I97">
-        <v>0.341016849235627</v>
+        <v>0.151309699487875</v>
       </c>
       <c r="J97">
-        <v>0.2320070314164575</v>
+        <v>0</v>
       </c>
       <c r="K97">
         <v>0</v>
@@ -6755,7 +6755,7 @@
         <v>0.2090209092421984</v>
       </c>
       <c r="N97">
-        <v>0.1929426790131443</v>
+        <v>0.05275291091015383</v>
       </c>
       <c r="O97">
         <v>0.7166666666666667</v>
@@ -6764,16 +6764,16 @@
         <v>0</v>
       </c>
       <c r="Q97">
-        <v>0.2503878600466827</v>
+        <v>0.2144344295664574</v>
       </c>
       <c r="R97">
-        <v>0.2014998601997285</v>
+        <v>0.1514809665465657</v>
       </c>
       <c r="S97">
-        <v>0.2802045847075085</v>
+        <v>0.2046423593843184</v>
       </c>
       <c r="T97">
-        <v>0.9047111147990098</v>
+        <v>0.03677816621792566</v>
       </c>
     </row>
     <row r="98" spans="1:20">
@@ -6843,13 +6843,13 @@
         <v>117</v>
       </c>
       <c r="B99">
-        <v>0.6757250788913208</v>
+        <v>0.5855376856598441</v>
       </c>
       <c r="C99" t="s">
         <v>136</v>
       </c>
       <c r="D99">
-        <v>1</v>
+        <v>0.9055555555555556</v>
       </c>
       <c r="E99">
         <v>0.620353584076456</v>
@@ -6858,19 +6858,19 @@
         <v>0.5</v>
       </c>
       <c r="G99">
-        <v>0.7126868770318362</v>
+        <v>0.6803410925474294</v>
       </c>
       <c r="H99">
-        <v>1</v>
+        <v>0.8300000000000001</v>
       </c>
       <c r="I99">
         <v>0.0916571623822173</v>
       </c>
       <c r="J99">
-        <v>0.9332363448065627</v>
+        <v>0.4379217079722647</v>
       </c>
       <c r="K99">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L99">
         <v>0.108840938941875</v>
@@ -6879,7 +6879,7 @@
         <v>0.4894756334860045</v>
       </c>
       <c r="N99">
-        <v>0.6564443436976306</v>
+        <v>0.5105149635595823</v>
       </c>
       <c r="O99">
         <v>1</v>
@@ -6888,13 +6888,13 @@
         <v>1</v>
       </c>
       <c r="Q99">
-        <v>0.5304464565849099</v>
+        <v>0.4930210303586446</v>
       </c>
       <c r="R99">
-        <v>0.762037375652808</v>
+        <v>0.5126731261740026</v>
       </c>
       <c r="S99">
-        <v>0.6387632807508055</v>
+        <v>0.4907342787722588</v>
       </c>
       <c r="T99">
         <v>0.971580507922511</v>
@@ -6967,7 +6967,7 @@
         <v>119</v>
       </c>
       <c r="B101">
-        <v>0.2880000980957226</v>
+        <v>0.2807396933030166</v>
       </c>
       <c r="C101" t="s">
         <v>135</v>
@@ -6988,7 +6988,7 @@
         <v>0</v>
       </c>
       <c r="I101">
-        <v>0.2566827452763405</v>
+        <v>0.2091790423121938</v>
       </c>
       <c r="J101">
         <v>0.05154648835437114</v>
@@ -7003,7 +7003,7 @@
         <v>0.8006406805404285</v>
       </c>
       <c r="N101">
-        <v>0.2696432347709606</v>
+        <v>0.2577866143857638</v>
       </c>
       <c r="O101">
         <v>0.2666666666666667</v>
@@ -7012,13 +7012,13 @@
         <v>0.325</v>
       </c>
       <c r="Q101">
-        <v>0.5384662872554845</v>
+        <v>0.5354255077284336</v>
       </c>
       <c r="R101">
-        <v>0.207212043565957</v>
+        <v>0.2066339293497064</v>
       </c>
       <c r="S101">
-        <v>0.1536336934712725</v>
+        <v>0.1391128838858607</v>
       </c>
       <c r="T101">
         <v>0.999999999999999</v>
@@ -7029,7 +7029,7 @@
         <v>120</v>
       </c>
       <c r="B102">
-        <v>0.1318699132961528</v>
+        <v>0.1316501605441191</v>
       </c>
       <c r="C102" t="s">
         <v>134</v>
@@ -7065,7 +7065,7 @@
         <v>0.3374307871805935</v>
       </c>
       <c r="N102">
-        <v>0.1506089337984506</v>
+        <v>0.1261365688698677</v>
       </c>
       <c r="O102">
         <v>0.5</v>
@@ -7074,16 +7074,16 @@
         <v>0</v>
       </c>
       <c r="Q102">
-        <v>0.1664656853034979</v>
+        <v>0.1601894393045736</v>
       </c>
       <c r="R102">
-        <v>0.1345783601465903</v>
+        <v>0.1333851177545045</v>
       </c>
       <c r="S102">
-        <v>0.2466155877476196</v>
+        <v>0.2461760822435521</v>
       </c>
       <c r="T102">
-        <v>0.2920974603874399</v>
+        <v>0.1784194920774879</v>
       </c>
     </row>
     <row r="103" spans="1:20">
@@ -7091,7 +7091,7 @@
         <v>121</v>
       </c>
       <c r="B103">
-        <v>0.0529573944279292</v>
+        <v>0.05244384265997586</v>
       </c>
       <c r="C103" t="s">
         <v>134</v>
@@ -7127,7 +7127,7 @@
         <v>0.1591957468445924</v>
       </c>
       <c r="N103">
-        <v>0.182322358764693</v>
+        <v>0.1251316016125671</v>
       </c>
       <c r="O103">
         <v>0</v>
@@ -7136,16 +7136,16 @@
         <v>0</v>
       </c>
       <c r="Q103">
-        <v>0.1138071865307403</v>
+        <v>0.099139897047318</v>
       </c>
       <c r="R103">
-        <v>0.05876089238832864</v>
+        <v>0.05597234146288479</v>
       </c>
       <c r="S103">
-        <v>0.1059147888558584</v>
+        <v>0.1048876853199517</v>
       </c>
       <c r="T103">
-        <v>0.185106431389838</v>
+        <v>0.1499999999999999</v>
       </c>
     </row>
     <row r="104" spans="1:20">
@@ -7153,7 +7153,7 @@
         <v>122</v>
       </c>
       <c r="B104">
-        <v>0.2787407600210989</v>
+        <v>0.1839283085331426</v>
       </c>
       <c r="C104" t="s">
         <v>135</v>
@@ -7165,31 +7165,31 @@
         <v>0.379646415923544</v>
       </c>
       <c r="F104">
-        <v>0.3928571428571429</v>
+        <v>0</v>
       </c>
       <c r="G104">
-        <v>0.2537603577764118</v>
+        <v>0.1307335520733248</v>
       </c>
       <c r="H104">
-        <v>0.5962500000000001</v>
+        <v>0.51125</v>
       </c>
       <c r="I104">
         <v>0</v>
       </c>
       <c r="J104">
-        <v>0.4741095325710248</v>
+        <v>0.4466186157266679</v>
       </c>
       <c r="K104">
-        <v>1</v>
+        <v>0.4333333333333333</v>
       </c>
       <c r="L104">
         <v>0.027086118117</v>
       </c>
       <c r="M104">
-        <v>0.5567592848453058</v>
+        <v>0.2627126002072336</v>
       </c>
       <c r="N104">
-        <v>0.3201265809667004</v>
+        <v>0.2727000994259131</v>
       </c>
       <c r="O104">
         <v>0</v>
@@ -7198,16 +7198,16 @@
         <v>0</v>
       </c>
       <c r="Q104">
-        <v>0.2481289668159541</v>
+        <v>0.1723971421951323</v>
       </c>
       <c r="R104">
-        <v>0.2896180393061621</v>
+        <v>0.1850711966721893</v>
       </c>
       <c r="S104">
-        <v>0.3037211622657859</v>
+        <v>0.2371230649929604</v>
       </c>
       <c r="T104">
-        <v>0.999999999999999</v>
+        <v>0.8579025396125589</v>
       </c>
     </row>
     <row r="105" spans="1:20">
@@ -7215,7 +7215,7 @@
         <v>123</v>
       </c>
       <c r="B105">
-        <v>0.216379046371097</v>
+        <v>0.2006770758047239</v>
       </c>
       <c r="C105" t="s">
         <v>135</v>
@@ -7236,13 +7236,13 @@
         <v>0.05</v>
       </c>
       <c r="I105">
-        <v>0.03978453215681071</v>
+        <v>0</v>
       </c>
       <c r="J105">
-        <v>0.687688303819106</v>
+        <v>0.6426216813895063</v>
       </c>
       <c r="K105">
-        <v>0.7166666666666667</v>
+        <v>0.4333333333333333</v>
       </c>
       <c r="L105">
         <v>0.0229138818825</v>
@@ -7251,7 +7251,7 @@
         <v>0.1224079851365004</v>
       </c>
       <c r="N105">
-        <v>0.4837862087341359</v>
+        <v>0.4463913798207021</v>
       </c>
       <c r="O105">
         <v>0.2666666666666667</v>
@@ -7260,16 +7260,16 @@
         <v>0.2375</v>
       </c>
       <c r="Q105">
-        <v>0.1620922198297914</v>
+        <v>0.1525018452978117</v>
       </c>
       <c r="R105">
-        <v>0.3505528585338215</v>
+        <v>0.2978253929900113</v>
       </c>
       <c r="S105">
-        <v>0.1576254181698358</v>
+        <v>0.1262214770370897</v>
       </c>
       <c r="T105">
-        <v>0.999999999999999</v>
+        <v>0.943161015845023</v>
       </c>
     </row>
     <row r="106" spans="1:20">
@@ -7277,34 +7277,34 @@
         <v>124</v>
       </c>
       <c r="B106">
-        <v>0.4872008309179287</v>
+        <v>0.2758361132448119</v>
       </c>
       <c r="C106" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="D106">
-        <v>0.4222222222222222</v>
+        <v>0</v>
       </c>
       <c r="E106">
-        <v>0.07798508700049113</v>
+        <v>0</v>
       </c>
       <c r="F106">
         <v>0.7571428571428571</v>
       </c>
       <c r="G106">
-        <v>0.4085655298930123</v>
+        <v>0.2371062073550404</v>
       </c>
       <c r="H106">
-        <v>0.89375</v>
+        <v>0.55375</v>
       </c>
       <c r="I106">
-        <v>0.2160118207468465</v>
+        <v>0.0145926440848958</v>
       </c>
       <c r="J106">
-        <v>0.9627477337068766</v>
+        <v>0.4794089717209908</v>
       </c>
       <c r="K106">
-        <v>0.7166666666666667</v>
+        <v>0</v>
       </c>
       <c r="L106">
         <v>0.5685538785463751</v>
@@ -7313,7 +7313,7 @@
         <v>0.5831730825364287</v>
       </c>
       <c r="N106">
-        <v>0.8040912940831074</v>
+        <v>0.4981015926765328</v>
       </c>
       <c r="O106">
         <v>0.2083333333333333</v>
@@ -7322,16 +7322,16 @@
         <v>0.325</v>
       </c>
       <c r="Q106">
-        <v>0.5143046816147776</v>
+        <v>0.4358297714551145</v>
       </c>
       <c r="R106">
-        <v>0.557684537382813</v>
+        <v>0.3452609104519636</v>
       </c>
       <c r="S106">
-        <v>0.5658361319428451</v>
+        <v>0.3145660191345835</v>
       </c>
       <c r="T106">
-        <v>0.999999999999999</v>
+        <v>0.6549125350595204</v>
       </c>
     </row>
     <row r="107" spans="1:20">
@@ -7339,7 +7339,7 @@
         <v>125</v>
       </c>
       <c r="B107">
-        <v>0.2106301196537562</v>
+        <v>0.1608121112146558</v>
       </c>
       <c r="C107" t="s">
         <v>135</v>
@@ -7357,13 +7357,13 @@
         <v>0.1651577840674002</v>
       </c>
       <c r="H107">
-        <v>0.35125</v>
+        <v>0.28125</v>
       </c>
       <c r="I107">
-        <v>0.274341166914134</v>
+        <v>0.03978849986889345</v>
       </c>
       <c r="J107">
-        <v>0.1841735239577585</v>
+        <v>0.1027802980693932</v>
       </c>
       <c r="K107">
         <v>0.1500000000000001</v>
@@ -7375,7 +7375,7 @@
         <v>0.06962306263125041</v>
       </c>
       <c r="N107">
-        <v>0.2283888864406418</v>
+        <v>0.2129910157115808</v>
       </c>
       <c r="O107">
         <v>0</v>
@@ -7384,16 +7384,16 @@
         <v>0.4125</v>
       </c>
       <c r="Q107">
-        <v>0.09470089430503811</v>
+        <v>0.09075191655657588</v>
       </c>
       <c r="R107">
-        <v>0.1558186315974726</v>
+        <v>0.1399181487598924</v>
       </c>
       <c r="S107">
-        <v>0.2561024552401121</v>
+        <v>0.1564664383619113</v>
       </c>
       <c r="T107">
-        <v>0.1734042875932253</v>
+        <v>0.1617021437966126</v>
       </c>
     </row>
     <row r="108" spans="1:20">
@@ -7401,7 +7401,7 @@
         <v>126</v>
       </c>
       <c r="B108">
-        <v>0.3446861215263722</v>
+        <v>0.2971700756998321</v>
       </c>
       <c r="C108" t="s">
         <v>135</v>
@@ -7419,16 +7419,16 @@
         <v>0.3272496350581542</v>
       </c>
       <c r="H108">
-        <v>0.715</v>
+        <v>0.6799999999999999</v>
       </c>
       <c r="I108">
-        <v>0.2220368990327404</v>
+        <v>0</v>
       </c>
       <c r="J108">
-        <v>0.1257735907639944</v>
+        <v>0.03534546451417322</v>
       </c>
       <c r="K108">
-        <v>0.1500000000000001</v>
+        <v>0</v>
       </c>
       <c r="L108">
         <v>0.108840938941875</v>
@@ -7437,7 +7437,7 @@
         <v>0.337225127598945</v>
       </c>
       <c r="N108">
-        <v>0.2936117702038186</v>
+        <v>0.1767326123527256</v>
       </c>
       <c r="O108">
         <v>0.3250000000000001</v>
@@ -7446,16 +7446,16 @@
         <v>0</v>
       </c>
       <c r="Q108">
-        <v>0.2487611477330111</v>
+        <v>0.2187860166428491</v>
       </c>
       <c r="R108">
-        <v>0.1600625862518162</v>
+        <v>0.11502391923077</v>
       </c>
       <c r="S108">
-        <v>0.3621226079945903</v>
+        <v>0.26709051634151</v>
       </c>
       <c r="T108">
-        <v>0.999999999999999</v>
+        <v>0.832826517191246</v>
       </c>
     </row>
     <row r="109" spans="1:20">
@@ -7525,7 +7525,7 @@
         <v>128</v>
       </c>
       <c r="B110">
-        <v>0.3698429186033866</v>
+        <v>0.3439811685621282</v>
       </c>
       <c r="C110" t="s">
         <v>135</v>
@@ -7549,7 +7549,7 @@
         <v>0.1509841300978179</v>
       </c>
       <c r="J110">
-        <v>0.5702170964294326</v>
+        <v>0.3860051530547435</v>
       </c>
       <c r="K110">
         <v>0.15</v>
@@ -7564,22 +7564,22 @@
         <v>0.4683245152759157</v>
       </c>
       <c r="O110">
-        <v>0.2666666666666667</v>
+        <v>0</v>
       </c>
       <c r="P110">
-        <v>0.575</v>
+        <v>0.3625</v>
       </c>
       <c r="Q110">
-        <v>0.3833978067980105</v>
+        <v>0.2276798696798975</v>
       </c>
       <c r="R110">
-        <v>0.3806185953428088</v>
+        <v>0.2401910639596437</v>
       </c>
       <c r="S110">
-        <v>0.4178280455480327</v>
+        <v>0.366104545465516</v>
       </c>
       <c r="T110">
-        <v>0.7400242908201713</v>
+        <v>0</v>
       </c>
     </row>
     <row r="111" spans="1:20">
@@ -7649,7 +7649,7 @@
         <v>130</v>
       </c>
       <c r="B112">
-        <v>0.01364240272473177</v>
+        <v>0.01311539791851239</v>
       </c>
       <c r="C112" t="s">
         <v>134</v>
@@ -7682,7 +7682,7 @@
         <v>0</v>
       </c>
       <c r="M112">
-        <v>0.06962306263125041</v>
+        <v>0</v>
       </c>
       <c r="N112">
         <v>0.04504181142414375</v>
@@ -7694,13 +7694,13 @@
         <v>0</v>
       </c>
       <c r="Q112">
-        <v>0.02660305427423139</v>
+        <v>0.01155153944296186</v>
       </c>
       <c r="R112">
-        <v>0.005057783287081576</v>
+        <v>0.002196183285287987</v>
       </c>
       <c r="S112">
-        <v>0.02728480544946353</v>
+        <v>0.02623079583702478</v>
       </c>
       <c r="T112">
         <v>0.1499999999999999</v>
@@ -7711,34 +7711,34 @@
         <v>131</v>
       </c>
       <c r="B113">
-        <v>0.7217994691446542</v>
+        <v>0.62722837347349</v>
       </c>
       <c r="C113" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="D113">
-        <v>1</v>
+        <v>0.9055555555555556</v>
       </c>
       <c r="E113">
-        <v>0.620353584076456</v>
+        <v>0.5183730856911983</v>
       </c>
       <c r="F113">
         <v>0.6357142857142857</v>
       </c>
       <c r="G113">
-        <v>0.7551870462747208</v>
+        <v>0.6877236569956524</v>
       </c>
       <c r="H113">
         <v>1</v>
       </c>
       <c r="I113">
-        <v>0.2730419982820105</v>
+        <v>0.06068328120882246</v>
       </c>
       <c r="J113">
-        <v>0.8881697223769631</v>
+        <v>0.754261506035002</v>
       </c>
       <c r="K113">
-        <v>1</v>
+        <v>0.15</v>
       </c>
       <c r="L113">
         <v>0.2305741207795</v>
@@ -7747,7 +7747,7 @@
         <v>0.7841759183366752</v>
       </c>
       <c r="N113">
-        <v>0.6776095574028846</v>
+        <v>0.590879269815797</v>
       </c>
       <c r="O113">
         <v>1</v>
@@ -7756,13 +7756,13 @@
         <v>0.7875</v>
       </c>
       <c r="Q113">
-        <v>0.5913754031520553</v>
+        <v>0.5691323292994652</v>
       </c>
       <c r="R113">
-        <v>0.7485071324318188</v>
+        <v>0.5918062659017218</v>
       </c>
       <c r="S113">
-        <v>0.6884118920145876</v>
+        <v>0.5667330899513277</v>
       </c>
       <c r="T113">
         <v>0.999999999999999</v>
@@ -7773,10 +7773,10 @@
         <v>132</v>
       </c>
       <c r="B114">
-        <v>0.5128635651219435</v>
+        <v>0.3754003424688841</v>
       </c>
       <c r="C114" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="D114">
         <v>0.7166666666666667</v>
@@ -7791,16 +7791,16 @@
         <v>0.4690253738497205</v>
       </c>
       <c r="H114">
-        <v>0.915</v>
+        <v>0.4475</v>
       </c>
       <c r="I114">
-        <v>0.3527580446079912</v>
+        <v>0.03292228035466767</v>
       </c>
       <c r="J114">
-        <v>0.3628648157565613</v>
+        <v>0.241527673157333</v>
       </c>
       <c r="K114">
-        <v>0.2666666666666667</v>
+        <v>0</v>
       </c>
       <c r="L114">
         <v>0.53717459191325</v>
@@ -7809,7 +7809,7 @@
         <v>0.7170930053829281</v>
       </c>
       <c r="N114">
-        <v>0.4197573439679279</v>
+        <v>0.3619211464210845</v>
       </c>
       <c r="O114">
         <v>0.2666666666666667</v>
@@ -7818,16 +7818,16 @@
         <v>0.4125</v>
       </c>
       <c r="Q114">
-        <v>0.5391762460969499</v>
+        <v>0.5243434253006892</v>
       </c>
       <c r="R114">
-        <v>0.4019968250420303</v>
+        <v>0.3365773851967953</v>
       </c>
       <c r="S114">
-        <v>0.5567017563941665</v>
+        <v>0.2817753110880476</v>
       </c>
       <c r="T114">
-        <v>0.3696073052917093</v>
+        <v>0</v>
       </c>
     </row>
     <row r="115" spans="1:20">
@@ -7835,7 +7835,7 @@
         <v>133</v>
       </c>
       <c r="B115">
-        <v>0.1259574643999848</v>
+        <v>0.03728969889130826</v>
       </c>
       <c r="C115" t="s">
         <v>134</v>
@@ -7847,16 +7847,16 @@
         <v>0.03599311707714975</v>
       </c>
       <c r="F115">
-        <v>0.35</v>
+        <v>0</v>
       </c>
       <c r="G115">
-        <v>0.1391243872221296</v>
+        <v>0.02951868759574299</v>
       </c>
       <c r="H115">
         <v>0</v>
       </c>
       <c r="I115">
-        <v>0.1847054465302821</v>
+        <v>0.07562383542532469</v>
       </c>
       <c r="J115">
         <v>0.07511013136381994</v>
@@ -7871,22 +7871,22 @@
         <v>0.100712374234342</v>
       </c>
       <c r="N115">
-        <v>0.2228269441698718</v>
+        <v>0.1027072486299612</v>
       </c>
       <c r="O115">
-        <v>0.575</v>
+        <v>0</v>
       </c>
       <c r="P115">
         <v>0.15</v>
       </c>
       <c r="Q115">
-        <v>0.07891935570981849</v>
+        <v>0.04811314794344812</v>
       </c>
       <c r="R115">
-        <v>0.1551825594434845</v>
+        <v>0.06049811392852678</v>
       </c>
       <c r="S115">
-        <v>0.1127905415778399</v>
+        <v>0.04506071018687352</v>
       </c>
       <c r="T115">
         <v>0.1249239775786869</v>

</xml_diff>